<commit_message>
Palletizado: mix como carga del camión con pallets unitarios por tipo
El escenario 5 reparte los pallets (o carros) enteros de cada tipo en el
vehículo según la producción de la semana pico, en vez de un pallet
promedio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/palletizado_PT.xlsx
+++ b/salida/palletizado_PT.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="178">
   <si>
     <t xml:space="preserve">General</t>
   </si>
@@ -368,18 +368,6 @@
     <t xml:space="preserve">Mes</t>
   </si>
   <si>
-    <t xml:space="preserve">Mix term. 2,5/5/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mix term. 25 a 100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mix cil. 2,5/5/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mix cil. 25 a 100</t>
-  </si>
-  <si>
     <t xml:space="preserve">Semana pico</t>
   </si>
   <si>
@@ -485,6 +473,9 @@
     <t xml:space="preserve">Unidades por pallet</t>
   </si>
   <si>
+    <t xml:space="preserve">por tipo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unidades por viaje</t>
   </si>
   <si>
@@ -506,6 +497,27 @@
     <t xml:space="preserve">%</t>
   </si>
   <si>
+    <t xml:space="preserve">5. Mix: pallets de cada tipo en el camión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pallets por semana (pico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pallets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pallets en el camión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidades en el camión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso en el camión</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rodantes (Master L3H2)</t>
   </si>
   <si>
@@ -522,6 +534,24 @@
   </si>
   <si>
     <t xml:space="preserve">5. Mix 25 a 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Mix: carros de cada tipo en el furgón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carros por semana (pico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carros en el furgón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ocupación del piso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso en el furgón</t>
   </si>
   <si>
     <t xml:space="preserve">Cilindros de manuales (sider)</t>
@@ -672,7 +702,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -743,6 +773,10 @@
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1822,11 +1856,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U36"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="2" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2728,7 +2762,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>113</v>
       </c>
@@ -2779,18 +2813,6 @@
       </c>
       <c r="Q23" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="R23" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="S23" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="T23" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="U23" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2861,22 +2883,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,1)/Datos!$C$4</f>
         <v>2.1675</v>
       </c>
-      <c r="R24" s="16" t="n">
-        <f aca="false">C24+D24+E24</f>
-        <v>1000.412131075</v>
-      </c>
-      <c r="S24" s="16" t="n">
-        <f aca="false">F24+G24+H24+I24</f>
-        <v>38.527995324125</v>
-      </c>
-      <c r="T24" s="16" t="n">
-        <f aca="false">K24+L24+M24</f>
-        <v>1039.875</v>
-      </c>
-      <c r="U24" s="16" t="n">
-        <f aca="false">N24+O24+P24+Q24</f>
-        <v>27.34875</v>
-      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
@@ -2946,22 +2952,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,2)/Datos!$C$4</f>
         <v>1.9125</v>
       </c>
-      <c r="R25" s="16" t="n">
-        <f aca="false">C25+D25+E25</f>
-        <v>800.32970486</v>
-      </c>
-      <c r="S25" s="16" t="n">
-        <f aca="false">F25+G25+H25+I25</f>
-        <v>33.995289991875</v>
-      </c>
-      <c r="T25" s="16" t="n">
-        <f aca="false">K25+L25+M25</f>
-        <v>831.9</v>
-      </c>
-      <c r="U25" s="16" t="n">
-        <f aca="false">N25+O25+P25+Q25</f>
-        <v>24.13125</v>
-      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
@@ -3031,22 +3021,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,3)/Datos!$C$4</f>
         <v>2.295</v>
       </c>
-      <c r="R26" s="16" t="n">
-        <f aca="false">C26+D26+E26</f>
-        <v>850.35031141375</v>
-      </c>
-      <c r="S26" s="16" t="n">
-        <f aca="false">F26+G26+H26+I26</f>
-        <v>40.79434799025</v>
-      </c>
-      <c r="T26" s="16" t="n">
-        <f aca="false">K26+L26+M26</f>
-        <v>883.89375</v>
-      </c>
-      <c r="U26" s="16" t="n">
-        <f aca="false">N26+O26+P26+Q26</f>
-        <v>28.9575</v>
-      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
@@ -3116,22 +3090,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,4)/Datos!$C$4</f>
         <v>2.295</v>
       </c>
-      <c r="R27" s="16" t="n">
-        <f aca="false">C27+D27+E27</f>
-        <v>850.35031141375</v>
-      </c>
-      <c r="S27" s="16" t="n">
-        <f aca="false">F27+G27+H27+I27</f>
-        <v>40.79434799025</v>
-      </c>
-      <c r="T27" s="16" t="n">
-        <f aca="false">K27+L27+M27</f>
-        <v>883.89375</v>
-      </c>
-      <c r="U27" s="16" t="n">
-        <f aca="false">N27+O27+P27+Q27</f>
-        <v>28.9575</v>
-      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
@@ -3201,22 +3159,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,5)/Datos!$C$4</f>
         <v>2.295</v>
       </c>
-      <c r="R28" s="16" t="n">
-        <f aca="false">C28+D28+E28</f>
-        <v>800.32970486</v>
-      </c>
-      <c r="S28" s="16" t="n">
-        <f aca="false">F28+G28+H28+I28</f>
-        <v>40.79434799025</v>
-      </c>
-      <c r="T28" s="16" t="n">
-        <f aca="false">K28+L28+M28</f>
-        <v>831.9</v>
-      </c>
-      <c r="U28" s="16" t="n">
-        <f aca="false">N28+O28+P28+Q28</f>
-        <v>28.9575</v>
-      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
@@ -3286,22 +3228,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,6)/Datos!$C$4</f>
         <v>2.04</v>
       </c>
-      <c r="R29" s="16" t="n">
-        <f aca="false">C29+D29+E29</f>
-        <v>750.30909830625</v>
-      </c>
-      <c r="S29" s="16" t="n">
-        <f aca="false">F29+G29+H29+I29</f>
-        <v>36.261642658</v>
-      </c>
-      <c r="T29" s="16" t="n">
-        <f aca="false">K29+L29+M29</f>
-        <v>779.90625</v>
-      </c>
-      <c r="U29" s="16" t="n">
-        <f aca="false">N29+O29+P29+Q29</f>
-        <v>25.74</v>
-      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
@@ -3371,22 +3297,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,7)/Datos!$C$4</f>
         <v>2.295</v>
       </c>
-      <c r="R30" s="16" t="n">
-        <f aca="false">C30+D30+E30</f>
-        <v>800.32970486</v>
-      </c>
-      <c r="S30" s="16" t="n">
-        <f aca="false">F30+G30+H30+I30</f>
-        <v>40.79434799025</v>
-      </c>
-      <c r="T30" s="16" t="n">
-        <f aca="false">K30+L30+M30</f>
-        <v>831.9</v>
-      </c>
-      <c r="U30" s="16" t="n">
-        <f aca="false">N30+O30+P30+Q30</f>
-        <v>28.9575</v>
-      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
@@ -3456,22 +3366,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,8)/Datos!$C$4</f>
         <v>2.295</v>
       </c>
-      <c r="R31" s="16" t="n">
-        <f aca="false">C31+D31+E31</f>
-        <v>800.32970486</v>
-      </c>
-      <c r="S31" s="16" t="n">
-        <f aca="false">F31+G31+H31+I31</f>
-        <v>40.79434799025</v>
-      </c>
-      <c r="T31" s="16" t="n">
-        <f aca="false">K31+L31+M31</f>
-        <v>831.9</v>
-      </c>
-      <c r="U31" s="16" t="n">
-        <f aca="false">N31+O31+P31+Q31</f>
-        <v>28.9575</v>
-      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
@@ -3541,22 +3435,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,9)/Datos!$C$4</f>
         <v>2.1675</v>
       </c>
-      <c r="R32" s="16" t="n">
-        <f aca="false">C32+D32+E32</f>
-        <v>800.32970486</v>
-      </c>
-      <c r="S32" s="16" t="n">
-        <f aca="false">F32+G32+H32+I32</f>
-        <v>38.527995324125</v>
-      </c>
-      <c r="T32" s="16" t="n">
-        <f aca="false">K32+L32+M32</f>
-        <v>831.9</v>
-      </c>
-      <c r="U32" s="16" t="n">
-        <f aca="false">N32+O32+P32+Q32</f>
-        <v>27.34875</v>
-      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
@@ -3626,22 +3504,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,10)/Datos!$C$4</f>
         <v>1.9125</v>
       </c>
-      <c r="R33" s="16" t="n">
-        <f aca="false">C33+D33+E33</f>
-        <v>750.30909830625</v>
-      </c>
-      <c r="S33" s="16" t="n">
-        <f aca="false">F33+G33+H33+I33</f>
-        <v>33.995289991875</v>
-      </c>
-      <c r="T33" s="16" t="n">
-        <f aca="false">K33+L33+M33</f>
-        <v>779.90625</v>
-      </c>
-      <c r="U33" s="16" t="n">
-        <f aca="false">N33+O33+P33+Q33</f>
-        <v>24.13125</v>
-      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
@@ -3711,22 +3573,6 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,11)/Datos!$C$4</f>
         <v>1.785</v>
       </c>
-      <c r="R34" s="16" t="n">
-        <f aca="false">C34+D34+E34</f>
-        <v>700.2884917525</v>
-      </c>
-      <c r="S34" s="16" t="n">
-        <f aca="false">F34+G34+H34+I34</f>
-        <v>31.72893732575</v>
-      </c>
-      <c r="T34" s="16" t="n">
-        <f aca="false">K34+L34+M34</f>
-        <v>727.9125</v>
-      </c>
-      <c r="U34" s="16" t="n">
-        <f aca="false">N34+O34+P34+Q34</f>
-        <v>22.5225</v>
-      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
@@ -3796,26 +3642,10 @@
         <f aca="false">Q$13*INDEX($B$18:$M$20,Q$14,12)/Datos!$C$4</f>
         <v>2.04</v>
       </c>
-      <c r="R35" s="16" t="n">
-        <f aca="false">C35+D35+E35</f>
-        <v>1100.4533441825</v>
-      </c>
-      <c r="S35" s="16" t="n">
-        <f aca="false">F35+G35+H35+I35</f>
-        <v>36.261642658</v>
-      </c>
-      <c r="T35" s="16" t="n">
-        <f aca="false">K35+L35+M35</f>
-        <v>1143.8625</v>
-      </c>
-      <c r="U35" s="16" t="n">
-        <f aca="false">N35+O35+P35+Q35</f>
-        <v>25.74</v>
-      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B36" s="13" t="n">
         <f aca="false">MAX(B24:B35)</f>
@@ -3880,22 +3710,6 @@
       <c r="Q36" s="13" t="n">
         <f aca="false">MAX(Q24:Q35)</f>
         <v>2.295</v>
-      </c>
-      <c r="R36" s="13" t="n">
-        <f aca="false">MAX(R24:R35)</f>
-        <v>1100.4533441825</v>
-      </c>
-      <c r="S36" s="13" t="n">
-        <f aca="false">MAX(S24:S35)</f>
-        <v>40.79434799025</v>
-      </c>
-      <c r="T36" s="13" t="n">
-        <f aca="false">MAX(T24:T35)</f>
-        <v>1143.8625</v>
-      </c>
-      <c r="U36" s="13" t="n">
-        <f aca="false">MAX(U24:U35)</f>
-        <v>28.9575</v>
       </c>
     </row>
   </sheetData>
@@ -3947,7 +3761,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>18</v>
@@ -3971,7 +3785,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>32</v>
@@ -3995,7 +3809,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>32</v>
@@ -4019,7 +3833,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>32</v>
@@ -4043,7 +3857,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>32</v>
@@ -4067,7 +3881,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>32</v>
@@ -4091,7 +3905,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>32</v>
@@ -4115,7 +3929,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>32</v>
@@ -4139,7 +3953,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>32</v>
@@ -4163,7 +3977,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>18</v>
@@ -4187,7 +4001,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>13</v>
@@ -4211,7 +4025,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4246,7 +4060,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B17" s="4" t="s">
         <v>32</v>
@@ -4286,7 +4100,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>32</v>
@@ -4326,7 +4140,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>32</v>
@@ -4366,7 +4180,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>32</v>
@@ -4406,7 +4220,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>32</v>
@@ -4446,7 +4260,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>32</v>
@@ -4486,7 +4300,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>32</v>
@@ -4526,7 +4340,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>18</v>
@@ -4566,7 +4380,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>13</v>
@@ -4630,7 +4444,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4644,7 +4458,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>32</v>
@@ -4656,7 +4470,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>32</v>
@@ -4668,7 +4482,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>32</v>
@@ -4680,7 +4494,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4703,7 +4517,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>32</v>
@@ -4727,7 +4541,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>32</v>
@@ -4751,7 +4565,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>32</v>
@@ -4775,7 +4589,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>32</v>
@@ -4799,7 +4613,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>32</v>
@@ -4823,7 +4637,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>32</v>
@@ -4861,7 +4675,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G124"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -4871,7 +4685,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4880,24 +4694,24 @@
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>32</v>
@@ -4918,14 +4732,13 @@
         <f aca="false">Pallet!F11</f>
         <v>60</v>
       </c>
-      <c r="G3" s="16" t="n">
-        <f aca="false">IF((IF(Pallet!D11=0,0,Produccion!C$13/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D$13/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E$13/Pallet!F11))=0,0,(Produccion!C$13+Produccion!D$13+Produccion!E$13)/(IF(Pallet!D11=0,0,Produccion!C$13/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D$13/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E$13/Pallet!F11)))</f>
-        <v>90.7491601395925</v>
+      <c r="G3" s="18" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>18</v>
@@ -4946,14 +4759,13 @@
         <f aca="false">Pallet!F12</f>
         <v>1038.8</v>
       </c>
-      <c r="G4" s="16" t="n">
-        <f aca="false">IF((IF(Pallet!D11=0,0,Produccion!C$13/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D$13/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E$13/Pallet!F11))=0,0,(Produccion!C$13/Pallet!D11*Pallet!D12+Produccion!D$13/Pallet!E11*Pallet!E12+Produccion!E$13/Pallet!F11*Pallet!F12)/(IF(Pallet!D11=0,0,Produccion!C$13/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D$13/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E$13/Pallet!F11)))</f>
-        <v>802.784630644483</v>
+      <c r="G4" s="18" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>32</v>
@@ -4975,13 +4787,13 @@
         <v>11</v>
       </c>
       <c r="G5" s="13" t="n">
-        <f aca="false">IF(G4=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/G4)))</f>
+        <f aca="false">$F$28</f>
         <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>32</v>
@@ -5003,13 +4815,13 @@
         <v>660</v>
       </c>
       <c r="G6" s="13" t="n">
-        <f aca="false">G5*G3</f>
-        <v>1270.4882419543</v>
+        <f aca="false">$F$29</f>
+        <v>1236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5017,7 +4829,7 @@
         <v>96</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C8" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B24/C$6)</f>
@@ -5036,7 +4848,7 @@
         <v>0.0697290939015152</v>
       </c>
       <c r="G8" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R24/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C24/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D24/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E24/Pallet!F11))/$F$28)</f>
         <v>0.787423368465136</v>
       </c>
     </row>
@@ -5045,7 +4857,7 @@
         <v>97</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C9" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B25/C$6)</f>
@@ -5064,7 +4876,7 @@
         <v>0.0557832751212121</v>
       </c>
       <c r="G9" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R25/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C25/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D25/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E25/Pallet!F11))/$F$28)</f>
         <v>0.629938694772109</v>
       </c>
     </row>
@@ -5073,7 +4885,7 @@
         <v>98</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C10" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B26/C$6)</f>
@@ -5092,7 +4904,7 @@
         <v>0.0592697298162879</v>
       </c>
       <c r="G10" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R26/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C26/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D26/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E26/Pallet!F11))/$F$28)</f>
         <v>0.669309863195366</v>
       </c>
     </row>
@@ -5101,7 +4913,7 @@
         <v>99</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C11" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B27/C$6)</f>
@@ -5120,7 +4932,7 @@
         <v>0.0592697298162879</v>
       </c>
       <c r="G11" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R27/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C27/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D27/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E27/Pallet!F11))/$F$28)</f>
         <v>0.669309863195366</v>
       </c>
     </row>
@@ -5129,7 +4941,7 @@
         <v>100</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C12" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B28/C$6)</f>
@@ -5148,7 +4960,7 @@
         <v>0.0557832751212121</v>
       </c>
       <c r="G12" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R28/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C28/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D28/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E28/Pallet!F11))/$F$28)</f>
         <v>0.629938694772109</v>
       </c>
     </row>
@@ -5157,7 +4969,7 @@
         <v>101</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C13" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B29/C$6)</f>
@@ -5176,7 +4988,7 @@
         <v>0.0522968204261364</v>
       </c>
       <c r="G13" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R29/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C29/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D29/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E29/Pallet!F11))/$F$28)</f>
         <v>0.590567526348852</v>
       </c>
     </row>
@@ -5185,7 +4997,7 @@
         <v>102</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C14" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B30/C$6)</f>
@@ -5204,7 +5016,7 @@
         <v>0.0557832751212121</v>
       </c>
       <c r="G14" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R30/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C30/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D30/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E30/Pallet!F11))/$F$28)</f>
         <v>0.629938694772109</v>
       </c>
     </row>
@@ -5213,7 +5025,7 @@
         <v>103</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C15" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B31/C$6)</f>
@@ -5232,7 +5044,7 @@
         <v>0.0557832751212121</v>
       </c>
       <c r="G15" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R31/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C31/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D31/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E31/Pallet!F11))/$F$28)</f>
         <v>0.629938694772109</v>
       </c>
     </row>
@@ -5241,7 +5053,7 @@
         <v>104</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C16" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B32/C$6)</f>
@@ -5260,7 +5072,7 @@
         <v>0.0557832751212121</v>
       </c>
       <c r="G16" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R32/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C32/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D32/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E32/Pallet!F11))/$F$28)</f>
         <v>0.629938694772109</v>
       </c>
     </row>
@@ -5269,7 +5081,7 @@
         <v>105</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C17" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B33/C$6)</f>
@@ -5288,7 +5100,7 @@
         <v>0.0522968204261364</v>
       </c>
       <c r="G17" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R33/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C33/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D33/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E33/Pallet!F11))/$F$28)</f>
         <v>0.590567526348852</v>
       </c>
     </row>
@@ -5297,7 +5109,7 @@
         <v>106</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C18" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B34/C$6)</f>
@@ -5316,7 +5128,7 @@
         <v>0.0488103657310606</v>
       </c>
       <c r="G18" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R34/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C34/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D34/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E34/Pallet!F11))/$F$28)</f>
         <v>0.551196357925595</v>
       </c>
     </row>
@@ -5325,7 +5137,7 @@
         <v>107</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C19" s="17" t="n">
         <f aca="false">IF(C$6=0,0,Produccion!B35/C$6)</f>
@@ -5344,70 +5156,70 @@
         <v>0.0767020032916667</v>
       </c>
       <c r="G19" s="17" t="n">
-        <f aca="false">IF(G$6=0,0,Produccion!R35/G$6)</f>
+        <f aca="false">IF($F$28=0,0,(IF(Pallet!D11=0,0,Produccion!C35/Pallet!D11)+IF(Pallet!E11=0,0,Produccion!D35/Pallet!E11)+IF(Pallet!F11=0,0,Produccion!E35/Pallet!F11))/$F$28)</f>
         <v>0.86616570531165</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C20" s="18" t="n">
+        <v>152</v>
+      </c>
+      <c r="C20" s="19" t="n">
         <f aca="false">MAX(C8:C19)</f>
         <v>0.19090856625</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="19" t="n">
         <f aca="false">MAX(D8:D19)</f>
         <v>0.086812758167517</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="19" t="n">
         <f aca="false">MAX(E8:E19)</f>
         <v>0.719087087414966</v>
       </c>
-      <c r="F20" s="18" t="n">
+      <c r="F20" s="19" t="n">
         <f aca="false">MAX(F8:F19)</f>
         <v>0.0767020032916667</v>
       </c>
-      <c r="G20" s="18" t="n">
+      <c r="G20" s="19" t="n">
         <f aca="false">MAX(G8:G19)</f>
         <v>0.86616570531165</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B21" s="4"/>
-      <c r="C21" s="19" t="str">
+      <c r="C21" s="20" t="str">
         <f aca="false">IF(C20=0,"-",IF(C20&gt;=1,ROUNDUP(C20,0)&amp;" por semana",IF(INT(1/C20)=1,"1 por semana","1 cada "&amp;INT(1/C20)&amp;" semanas")))</f>
         <v>1 cada 5 semanas</v>
       </c>
-      <c r="D21" s="19" t="str">
+      <c r="D21" s="20" t="str">
         <f aca="false">IF(D20=0,"-",IF(D20&gt;=1,ROUNDUP(D20,0)&amp;" por semana",IF(INT(1/D20)=1,"1 por semana","1 cada "&amp;INT(1/D20)&amp;" semanas")))</f>
         <v>1 cada 11 semanas</v>
       </c>
-      <c r="E21" s="19" t="str">
+      <c r="E21" s="20" t="str">
         <f aca="false">IF(E20=0,"-",IF(E20&gt;=1,ROUNDUP(E20,0)&amp;" por semana",IF(INT(1/E20)=1,"1 por semana","1 cada "&amp;INT(1/E20)&amp;" semanas")))</f>
         <v>1 por semana</v>
       </c>
-      <c r="F21" s="19" t="str">
+      <c r="F21" s="20" t="str">
         <f aca="false">IF(F20=0,"-",IF(F20&gt;=1,ROUNDUP(F20,0)&amp;" por semana",IF(INT(1/F20)=1,"1 por semana","1 cada "&amp;INT(1/F20)&amp;" semanas")))</f>
         <v>1 cada 13 semanas</v>
       </c>
-      <c r="G21" s="19" t="str">
+      <c r="G21" s="20" t="str">
         <f aca="false">IF(G20=0,"-",IF(G20&gt;=1,ROUNDUP(G20,0)&amp;" por semana",IF(INT(1/G20)=1,"1 por semana","1 cada "&amp;INT(1/G20)&amp;" semanas")))</f>
         <v>1 por semana</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C22" s="15" t="n">
         <f aca="false">IF(C20=0,0,IF(C20&gt;=1,C20/ROUNDUP(C20,0),C20*INT(1/C20)))</f>
@@ -5432,7 +5244,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5441,608 +5253,559 @@
         <v>2</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <f aca="false">IF(Pallet!D11=0,0,Produccion!C36/Pallet!D11)</f>
+        <v>1.21537861434524</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <f aca="false">IF(Pallet!E11=0,0,Produccion!D36/Pallet!E11)</f>
+        <v>10.0672192238095</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <f aca="false">IF(Pallet!F11=0,0,Produccion!E36/Pallet!F11)</f>
+        <v>0.843722036208333</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <f aca="false">SUM(C26:E26)</f>
+        <v>12.1263198743631</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <f aca="false">IF($F26=0,0,C26/$F26)</f>
+        <v>0.100226501274697</v>
+      </c>
+      <c r="D27" s="15" t="n">
+        <f aca="false">IF($F26=0,0,D26/$F26)</f>
+        <v>0.830195750080218</v>
+      </c>
+      <c r="E27" s="15" t="n">
+        <f aca="false">IF($F26=0,0,E26/$F26)</f>
+        <v>0.0695777486450849</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <f aca="false">SUM(C27:E27)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="B28" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C28" s="13" t="n">
+        <f aca="false">ROUND(SUM($C27:C27)*$F28,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D28" s="13" t="n">
+        <f aca="false">ROUND(SUM($C27:D27)*$F28,0)-ROUND(SUM($C27:C27)*$F28,0)</f>
+        <v>12</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <f aca="false">ROUND(SUM($C27:E27)*$F28,0)-ROUND(SUM($C27:D27)*$F28,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <f aca="false">IF(F26=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/(C27*Pallet!D12+D27*Pallet!E12+E27*Pallet!F12))))</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="B29" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="16" t="n">
+        <f aca="false">C28*Pallet!D11</f>
+        <v>168</v>
+      </c>
+      <c r="D29" s="16" t="n">
+        <f aca="false">D28*Pallet!E11</f>
+        <v>1008</v>
+      </c>
+      <c r="E29" s="16" t="n">
+        <f aca="false">E28*Pallet!F11</f>
+        <v>60</v>
+      </c>
+      <c r="F29" s="16" t="n">
+        <f aca="false">SUM(C29:E29)</f>
+        <v>1236</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="B30" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="16" t="n">
+        <f aca="false">C28*Pallet!D12</f>
+        <v>854.84</v>
+      </c>
+      <c r="D30" s="16" t="n">
+        <f aca="false">D28*Pallet!E12</f>
+        <v>9320.64</v>
+      </c>
+      <c r="E30" s="16" t="n">
+        <f aca="false">E28*Pallet!F12</f>
+        <v>1038.8</v>
+      </c>
+      <c r="F30" s="16" t="n">
+        <f aca="false">SUM(C30:E30)</f>
+        <v>11214.28</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="G25" s="2" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2"/>
+      <c r="B34" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="B26" s="4" t="s">
+      <c r="D34" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B35" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C26" s="13" t="n">
+      <c r="C35" s="13" t="n">
         <f aca="false">Camion!C14</f>
         <v>14</v>
       </c>
-      <c r="D26" s="13" t="n">
+      <c r="D35" s="13" t="n">
         <f aca="false">Camion!D14</f>
         <v>10</v>
       </c>
-      <c r="E26" s="13" t="n">
+      <c r="E35" s="13" t="n">
         <f aca="false">Camion!E14</f>
         <v>7</v>
       </c>
-      <c r="F26" s="13" t="n">
+      <c r="F35" s="13" t="n">
         <f aca="false">Camion!F14</f>
         <v>7</v>
       </c>
-      <c r="G26" s="13" t="n">
-        <f aca="false">IF((Produccion!F$13+Produccion!G$13+Produccion!H$13+Produccion!I$13)=0,0,MIN(INT((Produccion!F$13+Produccion!G$13+Produccion!H$13+Produccion!I$13)/(Produccion!F$13/Camion!C12+Produccion!G$13/Camion!D12+Produccion!H$13/Camion!E12+Produccion!I$13/Camion!F12)),INT(Datos!$C$51/((Produccion!F$13*Datos!$C$36+Produccion!G$13*Datos!$D$36+Produccion!H$13*Datos!$E$36+Produccion!I$13*Datos!$F$36)/(Produccion!F$13+Produccion!G$13+Produccion!H$13+Produccion!I$13)))))</f>
+      <c r="G35" s="13" t="n">
+        <f aca="false">$G$58</f>
         <v>9</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B27" s="4" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B36" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C27" s="13" t="n">
-        <f aca="false">C26</f>
+      <c r="C36" s="13" t="n">
+        <f aca="false">C35</f>
         <v>14</v>
       </c>
-      <c r="D27" s="13" t="n">
-        <f aca="false">D26</f>
+      <c r="D36" s="13" t="n">
+        <f aca="false">D35</f>
         <v>10</v>
       </c>
-      <c r="E27" s="13" t="n">
-        <f aca="false">E26</f>
+      <c r="E36" s="13" t="n">
+        <f aca="false">E35</f>
         <v>7</v>
       </c>
-      <c r="F27" s="13" t="n">
-        <f aca="false">F26</f>
+      <c r="F36" s="13" t="n">
+        <f aca="false">F35</f>
         <v>7</v>
       </c>
-      <c r="G27" s="13" t="n">
-        <f aca="false">G26</f>
+      <c r="G36" s="13" t="n">
+        <f aca="false">G35</f>
         <v>9</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C29" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F24/C$27)</f>
-        <v>0.687999916464286</v>
-      </c>
-      <c r="D29" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G24/D$27)</f>
-        <v>2.1190397428375</v>
-      </c>
-      <c r="E29" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H24/E$27)</f>
-        <v>0.66047992</v>
-      </c>
-      <c r="F29" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I24/F$27)</f>
-        <v>0.440319946464286</v>
-      </c>
-      <c r="G29" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S24/G$27)</f>
-        <v>4.28088836934722</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C30" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F25/C$27)</f>
-        <v>0.607058749821429</v>
-      </c>
-      <c r="D30" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G25/D$27)</f>
-        <v>1.8697409495625</v>
-      </c>
-      <c r="E30" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H25/E$27)</f>
-        <v>0.5827764</v>
-      </c>
-      <c r="F30" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I25/F$27)</f>
-        <v>0.388517599821429</v>
-      </c>
-      <c r="G30" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S25/G$27)</f>
-        <v>3.77725444354167</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C31" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F26/C$27)</f>
-        <v>0.728470499785714</v>
-      </c>
-      <c r="D31" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G26/D$27)</f>
-        <v>2.243689139475</v>
-      </c>
-      <c r="E31" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H26/E$27)</f>
-        <v>0.69933168</v>
-      </c>
-      <c r="F31" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I26/F$27)</f>
-        <v>0.466221119785714</v>
-      </c>
-      <c r="G31" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S26/G$27)</f>
-        <v>4.53270533225</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C32" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F27/C$27)</f>
-        <v>0.728470499785714</v>
-      </c>
-      <c r="D32" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G27/D$27)</f>
-        <v>2.243689139475</v>
-      </c>
-      <c r="E32" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H27/E$27)</f>
-        <v>0.69933168</v>
-      </c>
-      <c r="F32" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I27/F$27)</f>
-        <v>0.466221119785714</v>
-      </c>
-      <c r="G32" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S27/G$27)</f>
-        <v>4.53270533225</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C33" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F28/C$27)</f>
-        <v>0.728470499785714</v>
-      </c>
-      <c r="D33" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G28/D$27)</f>
-        <v>2.243689139475</v>
-      </c>
-      <c r="E33" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H28/E$27)</f>
-        <v>0.69933168</v>
-      </c>
-      <c r="F33" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I28/F$27)</f>
-        <v>0.466221119785714</v>
-      </c>
-      <c r="G33" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S28/G$27)</f>
-        <v>4.53270533225</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C34" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F29/C$27)</f>
-        <v>0.647529333142857</v>
-      </c>
-      <c r="D34" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G29/D$27)</f>
-        <v>1.9943903462</v>
-      </c>
-      <c r="E34" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H29/E$27)</f>
-        <v>0.62162816</v>
-      </c>
-      <c r="F34" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I29/F$27)</f>
-        <v>0.414418773142857</v>
-      </c>
-      <c r="G34" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S29/G$27)</f>
-        <v>4.02907140644444</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C35" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F30/C$27)</f>
-        <v>0.728470499785714</v>
-      </c>
-      <c r="D35" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G30/D$27)</f>
-        <v>2.243689139475</v>
-      </c>
-      <c r="E35" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H30/E$27)</f>
-        <v>0.69933168</v>
-      </c>
-      <c r="F35" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I30/F$27)</f>
-        <v>0.466221119785714</v>
-      </c>
-      <c r="G35" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S30/G$27)</f>
-        <v>4.53270533225</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C36" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F31/C$27)</f>
-        <v>0.728470499785714</v>
-      </c>
-      <c r="D36" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G31/D$27)</f>
-        <v>2.243689139475</v>
-      </c>
-      <c r="E36" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H31/E$27)</f>
-        <v>0.69933168</v>
-      </c>
-      <c r="F36" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I31/F$27)</f>
-        <v>0.466221119785714</v>
-      </c>
-      <c r="G36" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S31/G$27)</f>
-        <v>4.53270533225</v>
-      </c>
-    </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C37" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F32/C$27)</f>
-        <v>0.687999916464286</v>
-      </c>
-      <c r="D37" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G32/D$27)</f>
-        <v>2.1190397428375</v>
-      </c>
-      <c r="E37" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H32/E$27)</f>
-        <v>0.66047992</v>
-      </c>
-      <c r="F37" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I32/F$27)</f>
-        <v>0.440319946464286</v>
-      </c>
-      <c r="G37" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S32/G$27)</f>
-        <v>4.28088836934722</v>
+      <c r="A37" s="12" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C38" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F33/C$27)</f>
-        <v>0.607058749821429</v>
+        <f aca="false">IF(C$36=0,0,Produccion!F24/C$36)</f>
+        <v>0.687999916464286</v>
       </c>
       <c r="D38" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G33/D$27)</f>
-        <v>1.8697409495625</v>
+        <f aca="false">IF(D$36=0,0,Produccion!G24/D$36)</f>
+        <v>2.1190397428375</v>
       </c>
       <c r="E38" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H33/E$27)</f>
-        <v>0.5827764</v>
+        <f aca="false">IF(E$36=0,0,Produccion!H24/E$36)</f>
+        <v>0.66047992</v>
       </c>
       <c r="F38" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I33/F$27)</f>
-        <v>0.388517599821429</v>
+        <f aca="false">IF(F$36=0,0,Produccion!I24/F$36)</f>
+        <v>0.440319946464286</v>
       </c>
       <c r="G38" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S33/G$27)</f>
-        <v>3.77725444354167</v>
+        <f aca="false">IF($G$58=0,0,(Produccion!F24+Produccion!G24+Produccion!H24+Produccion!I24)/$G$58)</f>
+        <v>4.28088836934722</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C39" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F34/C$27)</f>
-        <v>0.5665881665</v>
+        <f aca="false">IF(C$36=0,0,Produccion!F25/C$36)</f>
+        <v>0.607058749821429</v>
       </c>
       <c r="D39" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G34/D$27)</f>
-        <v>1.745091552925</v>
+        <f aca="false">IF(D$36=0,0,Produccion!G25/D$36)</f>
+        <v>1.8697409495625</v>
       </c>
       <c r="E39" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H34/E$27)</f>
-        <v>0.54392464</v>
+        <f aca="false">IF(E$36=0,0,Produccion!H25/E$36)</f>
+        <v>0.5827764</v>
       </c>
       <c r="F39" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I34/F$27)</f>
-        <v>0.3626164265</v>
+        <f aca="false">IF(F$36=0,0,Produccion!I25/F$36)</f>
+        <v>0.388517599821429</v>
       </c>
       <c r="G39" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S34/G$27)</f>
-        <v>3.52543748063889</v>
+        <f aca="false">IF($G$58=0,0,(Produccion!F25+Produccion!G25+Produccion!H25+Produccion!I25)/$G$58)</f>
+        <v>3.77725444354167</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C40" s="17" t="n">
-        <f aca="false">IF(C$27=0,0,Produccion!F35/C$27)</f>
-        <v>0.647529333142857</v>
+        <f aca="false">IF(C$36=0,0,Produccion!F26/C$36)</f>
+        <v>0.728470499785714</v>
       </c>
       <c r="D40" s="17" t="n">
-        <f aca="false">IF(D$27=0,0,Produccion!G35/D$27)</f>
-        <v>1.9943903462</v>
+        <f aca="false">IF(D$36=0,0,Produccion!G26/D$36)</f>
+        <v>2.243689139475</v>
       </c>
       <c r="E40" s="17" t="n">
-        <f aca="false">IF(E$27=0,0,Produccion!H35/E$27)</f>
-        <v>0.62162816</v>
+        <f aca="false">IF(E$36=0,0,Produccion!H26/E$36)</f>
+        <v>0.69933168</v>
       </c>
       <c r="F40" s="17" t="n">
-        <f aca="false">IF(F$27=0,0,Produccion!I35/F$27)</f>
-        <v>0.414418773142857</v>
+        <f aca="false">IF(F$36=0,0,Produccion!I26/F$36)</f>
+        <v>0.466221119785714</v>
       </c>
       <c r="G40" s="17" t="n">
-        <f aca="false">IF(G$27=0,0,Produccion!S35/G$27)</f>
-        <v>4.02907140644444</v>
+        <f aca="false">IF($G$58=0,0,(Produccion!F26+Produccion!G26+Produccion!H26+Produccion!I26)/$G$58)</f>
+        <v>4.53270533225</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12" t="s">
-        <v>156</v>
+      <c r="A41" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C41" s="18" t="n">
-        <f aca="false">MAX(C29:C40)</f>
+        <v>152</v>
+      </c>
+      <c r="C41" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F27/C$36)</f>
         <v>0.728470499785714</v>
       </c>
-      <c r="D41" s="18" t="n">
-        <f aca="false">MAX(D29:D40)</f>
+      <c r="D41" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G27/D$36)</f>
         <v>2.243689139475</v>
       </c>
-      <c r="E41" s="18" t="n">
-        <f aca="false">MAX(E29:E40)</f>
+      <c r="E41" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H27/E$36)</f>
         <v>0.69933168</v>
       </c>
-      <c r="F41" s="18" t="n">
-        <f aca="false">MAX(F29:F40)</f>
+      <c r="F41" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I27/F$36)</f>
         <v>0.466221119785714</v>
       </c>
-      <c r="G41" s="18" t="n">
-        <f aca="false">MAX(G29:G40)</f>
+      <c r="G41" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F27+Produccion!G27+Produccion!H27+Produccion!I27)/$G$58)</f>
         <v>4.53270533225</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="B42" s="4"/>
-      <c r="C42" s="19" t="str">
-        <f aca="false">IF(C41=0,"-",IF(C41&gt;=1,ROUNDUP(C41,0)&amp;" por semana",IF(INT(1/C41)=1,"1 por semana","1 cada "&amp;INT(1/C41)&amp;" semanas")))</f>
-        <v>1 por semana</v>
-      </c>
-      <c r="D42" s="19" t="str">
-        <f aca="false">IF(D41=0,"-",IF(D41&gt;=1,ROUNDUP(D41,0)&amp;" por semana",IF(INT(1/D41)=1,"1 por semana","1 cada "&amp;INT(1/D41)&amp;" semanas")))</f>
-        <v>3 por semana</v>
-      </c>
-      <c r="E42" s="19" t="str">
-        <f aca="false">IF(E41=0,"-",IF(E41&gt;=1,ROUNDUP(E41,0)&amp;" por semana",IF(INT(1/E41)=1,"1 por semana","1 cada "&amp;INT(1/E41)&amp;" semanas")))</f>
-        <v>1 por semana</v>
-      </c>
-      <c r="F42" s="19" t="str">
-        <f aca="false">IF(F41=0,"-",IF(F41&gt;=1,ROUNDUP(F41,0)&amp;" por semana",IF(INT(1/F41)=1,"1 por semana","1 cada "&amp;INT(1/F41)&amp;" semanas")))</f>
-        <v>1 cada 2 semanas</v>
-      </c>
-      <c r="G42" s="19" t="str">
-        <f aca="false">IF(G41=0,"-",IF(G41&gt;=1,ROUNDUP(G41,0)&amp;" por semana",IF(INT(1/G41)=1,"1 por semana","1 cada "&amp;INT(1/G41)&amp;" semanas")))</f>
-        <v>5 por semana</v>
+      <c r="A42" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C42" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F28/C$36)</f>
+        <v>0.728470499785714</v>
+      </c>
+      <c r="D42" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G28/D$36)</f>
+        <v>2.243689139475</v>
+      </c>
+      <c r="E42" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H28/E$36)</f>
+        <v>0.69933168</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I28/F$36)</f>
+        <v>0.466221119785714</v>
+      </c>
+      <c r="G42" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F28+Produccion!G28+Produccion!H28+Produccion!I28)/$G$58)</f>
+        <v>4.53270533225</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>158</v>
+        <v>101</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C43" s="15" t="n">
-        <f aca="false">IF(C41=0,0,IF(C41&gt;=1,C41/ROUNDUP(C41,0),C41*INT(1/C41)))</f>
+        <v>152</v>
+      </c>
+      <c r="C43" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F29/C$36)</f>
+        <v>0.647529333142857</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G29/D$36)</f>
+        <v>1.9943903462</v>
+      </c>
+      <c r="E43" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H29/E$36)</f>
+        <v>0.62162816</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I29/F$36)</f>
+        <v>0.414418773142857</v>
+      </c>
+      <c r="G43" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F29+Produccion!G29+Produccion!H29+Produccion!I29)/$G$58)</f>
+        <v>4.02907140644444</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C44" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F30/C$36)</f>
         <v>0.728470499785714</v>
       </c>
-      <c r="D43" s="15" t="n">
-        <f aca="false">IF(D41=0,0,IF(D41&gt;=1,D41/ROUNDUP(D41,0),D41*INT(1/D41)))</f>
-        <v>0.747896379825</v>
-      </c>
-      <c r="E43" s="15" t="n">
-        <f aca="false">IF(E41=0,0,IF(E41&gt;=1,E41/ROUNDUP(E41,0),E41*INT(1/E41)))</f>
+      <c r="D44" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G30/D$36)</f>
+        <v>2.243689139475</v>
+      </c>
+      <c r="E44" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H30/E$36)</f>
         <v>0.69933168</v>
       </c>
-      <c r="F43" s="15" t="n">
-        <f aca="false">IF(F41=0,0,IF(F41&gt;=1,F41/ROUNDUP(F41,0),F41*INT(1/F41)))</f>
-        <v>0.932442239571429</v>
-      </c>
-      <c r="G43" s="15" t="n">
-        <f aca="false">IF(G41=0,0,IF(G41&gt;=1,G41/ROUNDUP(G41,0),G41*INT(1/G41)))</f>
-        <v>0.90654106645</v>
+      <c r="F44" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I30/F$36)</f>
+        <v>0.466221119785714</v>
+      </c>
+      <c r="G44" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F30+Produccion!G30+Produccion!H30+Produccion!I30)/$G$58)</f>
+        <v>4.53270533225</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
-        <v>166</v>
+      <c r="A45" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C45" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F31/C$36)</f>
+        <v>0.728470499785714</v>
+      </c>
+      <c r="D45" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G31/D$36)</f>
+        <v>2.243689139475</v>
+      </c>
+      <c r="E45" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H31/E$36)</f>
+        <v>0.69933168</v>
+      </c>
+      <c r="F45" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I31/F$36)</f>
+        <v>0.466221119785714</v>
+      </c>
+      <c r="G45" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F31+Produccion!G31+Produccion!H31+Produccion!I31)/$G$58)</f>
+        <v>4.53270533225</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>148</v>
-      </c>
-      <c r="E46" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>151</v>
+      <c r="A46" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C46" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F32/C$36)</f>
+        <v>0.687999916464286</v>
+      </c>
+      <c r="D46" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G32/D$36)</f>
+        <v>2.1190397428375</v>
+      </c>
+      <c r="E46" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H32/E$36)</f>
+        <v>0.66047992</v>
+      </c>
+      <c r="F46" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I32/F$36)</f>
+        <v>0.440319946464286</v>
+      </c>
+      <c r="G46" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F32+Produccion!G32+Produccion!H32+Produccion!I32)/$G$58)</f>
+        <v>4.28088836934722</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B47" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C47" s="16" t="n">
-        <f aca="false">Pallet!C23</f>
-        <v>780</v>
-      </c>
-      <c r="D47" s="16" t="n">
-        <f aca="false">Pallet!D23</f>
-        <v>288</v>
-      </c>
-      <c r="E47" s="16" t="n">
-        <f aca="false">Pallet!E23</f>
-        <v>126</v>
-      </c>
-      <c r="F47" s="16" t="n">
-        <f aca="false">Pallet!F23</f>
-        <v>60</v>
-      </c>
-      <c r="G47" s="16" t="n">
-        <f aca="false">IF((IF(Pallet!D23=0,0,Produccion!K$13/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L$13/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M$13/Pallet!F23))=0,0,(Produccion!K$13+Produccion!L$13+Produccion!M$13)/(IF(Pallet!D23=0,0,Produccion!K$13/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L$13/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M$13/Pallet!F23)))</f>
-        <v>130.841766623612</v>
+      <c r="C47" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F33/C$36)</f>
+        <v>0.607058749821429</v>
+      </c>
+      <c r="D47" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G33/D$36)</f>
+        <v>1.8697409495625</v>
+      </c>
+      <c r="E47" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H33/E$36)</f>
+        <v>0.5827764</v>
+      </c>
+      <c r="F47" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I33/F$36)</f>
+        <v>0.388517599821429</v>
+      </c>
+      <c r="G47" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F33+Produccion!G33+Produccion!H33+Produccion!I33)/$G$58)</f>
+        <v>3.77725444354167</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C48" s="16" t="n">
-        <f aca="false">Pallet!C24</f>
-        <v>630.8</v>
-      </c>
-      <c r="D48" s="16" t="n">
-        <f aca="false">Pallet!D24</f>
-        <v>464.24</v>
-      </c>
-      <c r="E48" s="16" t="n">
-        <f aca="false">Pallet!E24</f>
-        <v>387.68</v>
-      </c>
-      <c r="F48" s="16" t="n">
-        <f aca="false">Pallet!F24</f>
-        <v>365.6</v>
-      </c>
-      <c r="G48" s="16" t="n">
-        <f aca="false">IF((IF(Pallet!D23=0,0,Produccion!K$13/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L$13/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M$13/Pallet!F23))=0,0,(Produccion!K$13/Pallet!D23*Pallet!D24+Produccion!L$13/Pallet!E23*Pallet!E24+Produccion!M$13/Pallet!F23*Pallet!F24)/(IF(Pallet!D23=0,0,Produccion!K$13/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L$13/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M$13/Pallet!F23)))</f>
-        <v>390.928771653784</v>
+        <v>152</v>
+      </c>
+      <c r="C48" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F34/C$36)</f>
+        <v>0.5665881665</v>
+      </c>
+      <c r="D48" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G34/D$36)</f>
+        <v>1.745091552925</v>
+      </c>
+      <c r="E48" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H34/E$36)</f>
+        <v>0.54392464</v>
+      </c>
+      <c r="F48" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I34/F$36)</f>
+        <v>0.3626164265</v>
+      </c>
+      <c r="G48" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F34+Produccion!G34+Produccion!H34+Produccion!I34)/$G$58)</f>
+        <v>3.52543748063889</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12" t="s">
-        <v>138</v>
+      <c r="A49" s="3" t="s">
+        <v>107</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C49" s="13" t="n">
-        <f aca="false">IF(C48=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/C48)))</f>
-        <v>14</v>
-      </c>
-      <c r="D49" s="13" t="n">
-        <f aca="false">IF(D48=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/D48)))</f>
-        <v>14</v>
-      </c>
-      <c r="E49" s="13" t="n">
-        <f aca="false">IF(E48=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/E48)))</f>
-        <v>14</v>
-      </c>
-      <c r="F49" s="13" t="n">
-        <f aca="false">IF(F48=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/F48)))</f>
-        <v>14</v>
-      </c>
-      <c r="G49" s="13" t="n">
-        <f aca="false">IF(G48=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/G48)))</f>
-        <v>14</v>
+        <v>152</v>
+      </c>
+      <c r="C49" s="17" t="n">
+        <f aca="false">IF(C$36=0,0,Produccion!F35/C$36)</f>
+        <v>0.647529333142857</v>
+      </c>
+      <c r="D49" s="17" t="n">
+        <f aca="false">IF(D$36=0,0,Produccion!G35/D$36)</f>
+        <v>1.9943903462</v>
+      </c>
+      <c r="E49" s="17" t="n">
+        <f aca="false">IF(E$36=0,0,Produccion!H35/E$36)</f>
+        <v>0.62162816</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <f aca="false">IF(F$36=0,0,Produccion!I35/F$36)</f>
+        <v>0.414418773142857</v>
+      </c>
+      <c r="G49" s="17" t="n">
+        <f aca="false">IF($G$58=0,0,(Produccion!F35+Produccion!G35+Produccion!H35+Produccion!I35)/$G$58)</f>
+        <v>4.02907140644444</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6050,1011 +5813,1674 @@
         <v>153</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C50" s="13" t="n">
-        <f aca="false">C49*C47</f>
-        <v>10920</v>
-      </c>
-      <c r="D50" s="13" t="n">
-        <f aca="false">D49*D47</f>
-        <v>4032</v>
-      </c>
-      <c r="E50" s="13" t="n">
-        <f aca="false">E49*E47</f>
-        <v>1764</v>
-      </c>
-      <c r="F50" s="13" t="n">
-        <f aca="false">F49*F47</f>
-        <v>840</v>
-      </c>
-      <c r="G50" s="13" t="n">
-        <f aca="false">G49*G47</f>
-        <v>1831.78473273057</v>
+        <v>152</v>
+      </c>
+      <c r="C50" s="19" t="n">
+        <f aca="false">MAX(C38:C49)</f>
+        <v>0.728470499785714</v>
+      </c>
+      <c r="D50" s="19" t="n">
+        <f aca="false">MAX(D38:D49)</f>
+        <v>2.243689139475</v>
+      </c>
+      <c r="E50" s="19" t="n">
+        <f aca="false">MAX(E38:E49)</f>
+        <v>0.69933168</v>
+      </c>
+      <c r="F50" s="19" t="n">
+        <f aca="false">MAX(F38:F49)</f>
+        <v>0.466221119785714</v>
+      </c>
+      <c r="G50" s="19" t="n">
+        <f aca="false">MAX(G38:G49)</f>
+        <v>4.53270533225</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
         <v>154</v>
       </c>
+      <c r="B51" s="4"/>
+      <c r="C51" s="20" t="str">
+        <f aca="false">IF(C50=0,"-",IF(C50&gt;=1,ROUNDUP(C50,0)&amp;" por semana",IF(INT(1/C50)=1,"1 por semana","1 cada "&amp;INT(1/C50)&amp;" semanas")))</f>
+        <v>1 por semana</v>
+      </c>
+      <c r="D51" s="20" t="str">
+        <f aca="false">IF(D50=0,"-",IF(D50&gt;=1,ROUNDUP(D50,0)&amp;" por semana",IF(INT(1/D50)=1,"1 por semana","1 cada "&amp;INT(1/D50)&amp;" semanas")))</f>
+        <v>3 por semana</v>
+      </c>
+      <c r="E51" s="20" t="str">
+        <f aca="false">IF(E50=0,"-",IF(E50&gt;=1,ROUNDUP(E50,0)&amp;" por semana",IF(INT(1/E50)=1,"1 por semana","1 cada "&amp;INT(1/E50)&amp;" semanas")))</f>
+        <v>1 por semana</v>
+      </c>
+      <c r="F51" s="20" t="str">
+        <f aca="false">IF(F50=0,"-",IF(F50&gt;=1,ROUNDUP(F50,0)&amp;" por semana",IF(INT(1/F50)=1,"1 por semana","1 cada "&amp;INT(1/F50)&amp;" semanas")))</f>
+        <v>1 cada 2 semanas</v>
+      </c>
+      <c r="G51" s="20" t="str">
+        <f aca="false">IF(G50=0,"-",IF(G50&gt;=1,ROUNDUP(G50,0)&amp;" por semana",IF(INT(1/G50)=1,"1 por semana","1 cada "&amp;INT(1/G50)&amp;" semanas")))</f>
+        <v>5 por semana</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>96</v>
+        <v>155</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C52" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J24/C$50)</f>
-        <v>0.468538461538462</v>
-      </c>
-      <c r="D52" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K24/D$50)</f>
-        <v>0.0413504464285714</v>
-      </c>
-      <c r="E52" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L24/E$50)</f>
-        <v>0.466482426303855</v>
-      </c>
-      <c r="F52" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M24/F$50)</f>
-        <v>0.0598511904761905</v>
-      </c>
-      <c r="G52" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T24/G$50)</f>
-        <v>0.567684063208617</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C53" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J25/C$50)</f>
-        <v>0.351403846153846</v>
-      </c>
-      <c r="D53" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K25/D$50)</f>
-        <v>0.0330803571428571</v>
-      </c>
-      <c r="E53" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L25/E$50)</f>
-        <v>0.373185941043084</v>
-      </c>
-      <c r="F53" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M25/F$50)</f>
-        <v>0.0478809523809524</v>
-      </c>
-      <c r="G53" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T25/G$50)</f>
-        <v>0.454147250566894</v>
+        <v>156</v>
+      </c>
+      <c r="C52" s="15" t="n">
+        <f aca="false">IF(C50=0,0,IF(C50&gt;=1,C50/ROUNDUP(C50,0),C50*INT(1/C50)))</f>
+        <v>0.728470499785714</v>
+      </c>
+      <c r="D52" s="15" t="n">
+        <f aca="false">IF(D50=0,0,IF(D50&gt;=1,D50/ROUNDUP(D50,0),D50*INT(1/D50)))</f>
+        <v>0.747896379825</v>
+      </c>
+      <c r="E52" s="15" t="n">
+        <f aca="false">IF(E50=0,0,IF(E50&gt;=1,E50/ROUNDUP(E50,0),E50*INT(1/E50)))</f>
+        <v>0.69933168</v>
+      </c>
+      <c r="F52" s="15" t="n">
+        <f aca="false">IF(F50=0,0,IF(F50&gt;=1,F50/ROUNDUP(F50,0),F50*INT(1/F50)))</f>
+        <v>0.932442239571429</v>
+      </c>
+      <c r="G52" s="15" t="n">
+        <f aca="false">IF(G50=0,0,IF(G50&gt;=1,G50/ROUNDUP(G50,0),G50*INT(1/G50)))</f>
+        <v>0.90654106645</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C54" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J26/C$50)</f>
-        <v>0.312358974358974</v>
-      </c>
-      <c r="D54" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K26/D$50)</f>
-        <v>0.0351478794642857</v>
-      </c>
-      <c r="E54" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L26/E$50)</f>
-        <v>0.396510062358277</v>
-      </c>
-      <c r="F54" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M26/F$50)</f>
-        <v>0.0508735119047619</v>
-      </c>
-      <c r="G54" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T26/G$50)</f>
-        <v>0.482531453727324</v>
+      <c r="A54" s="1" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C55" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J27/C$50)</f>
-        <v>0.292836538461538</v>
-      </c>
-      <c r="D55" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K27/D$50)</f>
-        <v>0.0351478794642857</v>
-      </c>
-      <c r="E55" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L27/E$50)</f>
-        <v>0.396510062358277</v>
-      </c>
-      <c r="F55" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M27/F$50)</f>
-        <v>0.0508735119047619</v>
-      </c>
-      <c r="G55" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T27/G$50)</f>
-        <v>0.482531453727324</v>
+      <c r="A55" s="2"/>
+      <c r="B55" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>100</v>
+        <v>171</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="C56" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J28/C$50)</f>
-        <v>0.273314102564103</v>
+        <f aca="false">Produccion!F36</f>
+        <v>10.198586997</v>
       </c>
       <c r="D56" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K28/D$50)</f>
-        <v>0.0330803571428571</v>
+        <f aca="false">Produccion!G36</f>
+        <v>22.43689139475</v>
       </c>
       <c r="E56" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L28/E$50)</f>
-        <v>0.373185941043084</v>
+        <f aca="false">Produccion!H36</f>
+        <v>4.89532176</v>
       </c>
       <c r="F56" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M28/F$50)</f>
-        <v>0.0478809523809524</v>
+        <f aca="false">Produccion!I36</f>
+        <v>3.2635478385</v>
       </c>
       <c r="G56" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T28/G$50)</f>
-        <v>0.454147250566894</v>
+        <f aca="false">SUM(C56:F56)</f>
+        <v>40.79434799025</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
-        <v>101</v>
+        <v>160</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C57" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J29/C$50)</f>
-        <v>0.273314102564103</v>
-      </c>
-      <c r="D57" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K29/D$50)</f>
-        <v>0.0310128348214286</v>
-      </c>
-      <c r="E57" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L29/E$50)</f>
-        <v>0.349861819727891</v>
-      </c>
-      <c r="F57" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M29/F$50)</f>
-        <v>0.0448883928571429</v>
-      </c>
-      <c r="G57" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T29/G$50)</f>
-        <v>0.425763047406463</v>
+        <v>156</v>
+      </c>
+      <c r="C57" s="15" t="n">
+        <f aca="false">IF($G56=0,0,C56/$G56)</f>
+        <v>0.249999999986211</v>
+      </c>
+      <c r="D57" s="15" t="n">
+        <f aca="false">IF($G56=0,0,D56/$G56)</f>
+        <v>0.550000000002758</v>
+      </c>
+      <c r="E57" s="15" t="n">
+        <f aca="false">IF($G56=0,0,E56/$G56)</f>
+        <v>0.12000000002868</v>
+      </c>
+      <c r="F57" s="15" t="n">
+        <f aca="false">IF($G56=0,0,F56/$G56)</f>
+        <v>0.0799999999823505</v>
+      </c>
+      <c r="G57" s="15" t="n">
+        <f aca="false">SUM(C57:F57)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3" t="s">
-        <v>102</v>
+      <c r="A58" s="12" t="s">
+        <v>173</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C58" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J30/C$50)</f>
-        <v>0.292836538461538</v>
-      </c>
-      <c r="D58" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K30/D$50)</f>
-        <v>0.0330803571428571</v>
-      </c>
-      <c r="E58" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L30/E$50)</f>
-        <v>0.373185941043084</v>
-      </c>
-      <c r="F58" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M30/F$50)</f>
-        <v>0.0478809523809524</v>
-      </c>
-      <c r="G58" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T30/G$50)</f>
-        <v>0.454147250566894</v>
+        <v>172</v>
+      </c>
+      <c r="C58" s="13" t="n">
+        <f aca="false">ROUND(SUM($C57:C57)*$G58,0)</f>
+        <v>2</v>
+      </c>
+      <c r="D58" s="13" t="n">
+        <f aca="false">ROUND(SUM($C57:D57)*$G58,0)-ROUND(SUM($C57:C57)*$G58,0)</f>
+        <v>5</v>
+      </c>
+      <c r="E58" s="13" t="n">
+        <f aca="false">ROUND(SUM($C57:E57)*$G58,0)-ROUND(SUM($C57:D57)*$G58,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F58" s="13" t="n">
+        <f aca="false">ROUND(SUM($C57:F57)*$G58,0)-ROUND(SUM($C57:E57)*$G58,0)</f>
+        <v>1</v>
+      </c>
+      <c r="G58" s="13" t="n">
+        <f aca="false">IF(G56=0,0,MIN(INT(1/(C57/Camion!C12+D57/Camion!D12+E57/Camion!E12+F57/Camion!F12)),INT(Datos!$C$51/(C57*Datos!$C$36+D57*Datos!$D$36+E57*Datos!$E$36+F57*Datos!$F$36))))</f>
+        <v>9</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>103</v>
+        <v>174</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C59" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J31/C$50)</f>
-        <v>0.292836538461538</v>
-      </c>
-      <c r="D59" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K31/D$50)</f>
-        <v>0.0330803571428571</v>
-      </c>
-      <c r="E59" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L31/E$50)</f>
-        <v>0.373185941043084</v>
-      </c>
-      <c r="F59" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M31/F$50)</f>
-        <v>0.0478809523809524</v>
-      </c>
-      <c r="G59" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T31/G$50)</f>
-        <v>0.454147250566894</v>
+        <v>156</v>
+      </c>
+      <c r="C59" s="15" t="n">
+        <f aca="false">IF(Camion!C12=0,0,C58/Camion!C12)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="D59" s="15" t="n">
+        <f aca="false">IF(Camion!D12=0,0,D58/Camion!D12)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E59" s="15" t="n">
+        <f aca="false">IF(Camion!E12=0,0,E58/Camion!E12)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="F59" s="15" t="n">
+        <f aca="false">IF(Camion!F12=0,0,F58/Camion!F12)</f>
+        <v>0.142857142857143</v>
+      </c>
+      <c r="G59" s="15" t="n">
+        <f aca="false">SUM(C59:F59)</f>
+        <v>0.928571428571429</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>104</v>
+        <v>175</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C60" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J32/C$50)</f>
-        <v>0.292836538461538</v>
-      </c>
-      <c r="D60" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K32/D$50)</f>
-        <v>0.0330803571428571</v>
-      </c>
-      <c r="E60" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L32/E$50)</f>
-        <v>0.373185941043084</v>
-      </c>
-      <c r="F60" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M32/F$50)</f>
-        <v>0.0478809523809524</v>
-      </c>
-      <c r="G60" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T32/G$50)</f>
-        <v>0.454147250566894</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C61" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J33/C$50)</f>
-        <v>0.292836538461538</v>
-      </c>
-      <c r="D61" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K33/D$50)</f>
-        <v>0.0310128348214286</v>
-      </c>
-      <c r="E61" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L33/E$50)</f>
-        <v>0.349861819727891</v>
-      </c>
-      <c r="F61" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M33/F$50)</f>
-        <v>0.0448883928571429</v>
-      </c>
-      <c r="G61" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T33/G$50)</f>
-        <v>0.425763047406463</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C62" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J34/C$50)</f>
-        <v>0.292836538461538</v>
-      </c>
-      <c r="D62" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K34/D$50)</f>
-        <v>0.0289453125</v>
-      </c>
-      <c r="E62" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L34/E$50)</f>
-        <v>0.326537698412698</v>
-      </c>
-      <c r="F62" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M34/F$50)</f>
-        <v>0.0418958333333333</v>
-      </c>
-      <c r="G62" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T34/G$50)</f>
-        <v>0.397378844246032</v>
+        <v>18</v>
+      </c>
+      <c r="C60" s="16" t="n">
+        <f aca="false">C58*Datos!$C$36</f>
+        <v>110</v>
+      </c>
+      <c r="D60" s="16" t="n">
+        <f aca="false">D58*Datos!$D$36</f>
+        <v>500</v>
+      </c>
+      <c r="E60" s="16" t="n">
+        <f aca="false">E58*Datos!$E$36</f>
+        <v>140</v>
+      </c>
+      <c r="F60" s="16" t="n">
+        <f aca="false">F58*Datos!$F$36</f>
+        <v>185</v>
+      </c>
+      <c r="G60" s="16" t="n">
+        <f aca="false">SUM(C60:F60)</f>
+        <v>935</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C63" s="17" t="n">
-        <f aca="false">IF(C$50=0,0,Produccion!J35/C$50)</f>
-        <v>0.468538461538462</v>
-      </c>
-      <c r="D63" s="17" t="n">
-        <f aca="false">IF(D$50=0,0,Produccion!K35/D$50)</f>
-        <v>0.0454854910714286</v>
-      </c>
-      <c r="E63" s="17" t="n">
-        <f aca="false">IF(E$50=0,0,Produccion!L35/E$50)</f>
-        <v>0.51313066893424</v>
-      </c>
-      <c r="F63" s="17" t="n">
-        <f aca="false">IF(F$50=0,0,Produccion!M35/F$50)</f>
-        <v>0.0658363095238095</v>
-      </c>
-      <c r="G63" s="17" t="n">
-        <f aca="false">IF(G$50=0,0,Produccion!T35/G$50)</f>
-        <v>0.624452469529478</v>
+      <c r="A63" s="1" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C64" s="18" t="n">
-        <f aca="false">MAX(C52:C63)</f>
-        <v>0.468538461538462</v>
-      </c>
-      <c r="D64" s="18" t="n">
-        <f aca="false">MAX(D52:D63)</f>
-        <v>0.0454854910714286</v>
-      </c>
-      <c r="E64" s="18" t="n">
-        <f aca="false">MAX(E52:E63)</f>
-        <v>0.51313066893424</v>
-      </c>
-      <c r="F64" s="18" t="n">
-        <f aca="false">MAX(F52:F63)</f>
-        <v>0.0658363095238095</v>
-      </c>
-      <c r="G64" s="18" t="n">
-        <f aca="false">MAX(G52:G63)</f>
-        <v>0.624452469529478</v>
+      <c r="A64" s="2"/>
+      <c r="B64" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="B65" s="4"/>
-      <c r="C65" s="19" t="str">
-        <f aca="false">IF(C64=0,"-",IF(C64&gt;=1,ROUNDUP(C64,0)&amp;" por semana",IF(INT(1/C64)=1,"1 por semana","1 cada "&amp;INT(1/C64)&amp;" semanas")))</f>
-        <v>1 cada 2 semanas</v>
-      </c>
-      <c r="D65" s="19" t="str">
-        <f aca="false">IF(D64=0,"-",IF(D64&gt;=1,ROUNDUP(D64,0)&amp;" por semana",IF(INT(1/D64)=1,"1 por semana","1 cada "&amp;INT(1/D64)&amp;" semanas")))</f>
-        <v>1 cada 21 semanas</v>
-      </c>
-      <c r="E65" s="19" t="str">
-        <f aca="false">IF(E64=0,"-",IF(E64&gt;=1,ROUNDUP(E64,0)&amp;" por semana",IF(INT(1/E64)=1,"1 por semana","1 cada "&amp;INT(1/E64)&amp;" semanas")))</f>
-        <v>1 por semana</v>
-      </c>
-      <c r="F65" s="19" t="str">
-        <f aca="false">IF(F64=0,"-",IF(F64&gt;=1,ROUNDUP(F64,0)&amp;" por semana",IF(INT(1/F64)=1,"1 por semana","1 cada "&amp;INT(1/F64)&amp;" semanas")))</f>
-        <v>1 cada 15 semanas</v>
-      </c>
-      <c r="G65" s="19" t="str">
-        <f aca="false">IF(G64=0,"-",IF(G64&gt;=1,ROUNDUP(G64,0)&amp;" por semana",IF(INT(1/G64)=1,"1 por semana","1 cada "&amp;INT(1/G64)&amp;" semanas")))</f>
-        <v>1 por semana</v>
+      <c r="A65" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C65" s="16" t="n">
+        <f aca="false">Pallet!C23</f>
+        <v>780</v>
+      </c>
+      <c r="D65" s="16" t="n">
+        <f aca="false">Pallet!D23</f>
+        <v>288</v>
+      </c>
+      <c r="E65" s="16" t="n">
+        <f aca="false">Pallet!E23</f>
+        <v>126</v>
+      </c>
+      <c r="F65" s="16" t="n">
+        <f aca="false">Pallet!F23</f>
+        <v>60</v>
+      </c>
+      <c r="G65" s="18" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>158</v>
+        <v>124</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C66" s="15" t="n">
-        <f aca="false">IF(C64=0,0,IF(C64&gt;=1,C64/ROUNDUP(C64,0),C64*INT(1/C64)))</f>
-        <v>0.937076923076923</v>
-      </c>
-      <c r="D66" s="15" t="n">
-        <f aca="false">IF(D64=0,0,IF(D64&gt;=1,D64/ROUNDUP(D64,0),D64*INT(1/D64)))</f>
-        <v>0.9551953125</v>
-      </c>
-      <c r="E66" s="15" t="n">
-        <f aca="false">IF(E64=0,0,IF(E64&gt;=1,E64/ROUNDUP(E64,0),E64*INT(1/E64)))</f>
-        <v>0.51313066893424</v>
-      </c>
-      <c r="F66" s="15" t="n">
-        <f aca="false">IF(F64=0,0,IF(F64&gt;=1,F64/ROUNDUP(F64,0),F64*INT(1/F64)))</f>
-        <v>0.987544642857143</v>
-      </c>
-      <c r="G66" s="15" t="n">
-        <f aca="false">IF(G64=0,0,IF(G64&gt;=1,G64/ROUNDUP(G64,0),G64*INT(1/G64)))</f>
-        <v>0.624452469529478</v>
+        <v>18</v>
+      </c>
+      <c r="C66" s="16" t="n">
+        <f aca="false">Pallet!C24</f>
+        <v>630.8</v>
+      </c>
+      <c r="D66" s="16" t="n">
+        <f aca="false">Pallet!D24</f>
+        <v>464.24</v>
+      </c>
+      <c r="E66" s="16" t="n">
+        <f aca="false">Pallet!E24</f>
+        <v>387.68</v>
+      </c>
+      <c r="F66" s="16" t="n">
+        <f aca="false">Pallet!F24</f>
+        <v>365.6</v>
+      </c>
+      <c r="G66" s="18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C67" s="13" t="n">
+        <f aca="false">IF(C66=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/C66)))</f>
+        <v>14</v>
+      </c>
+      <c r="D67" s="13" t="n">
+        <f aca="false">IF(D66=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/D66)))</f>
+        <v>14</v>
+      </c>
+      <c r="E67" s="13" t="n">
+        <f aca="false">IF(E66=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/E66)))</f>
+        <v>14</v>
+      </c>
+      <c r="F67" s="13" t="n">
+        <f aca="false">IF(F66=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/F66)))</f>
+        <v>14</v>
+      </c>
+      <c r="G67" s="13" t="n">
+        <f aca="false">$F$90</f>
+        <v>14</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="1" t="s">
-        <v>167</v>
+      <c r="A68" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C68" s="13" t="n">
+        <f aca="false">C67*C65</f>
+        <v>10920</v>
+      </c>
+      <c r="D68" s="13" t="n">
+        <f aca="false">D67*D65</f>
+        <v>4032</v>
+      </c>
+      <c r="E68" s="13" t="n">
+        <f aca="false">E67*E65</f>
+        <v>1764</v>
+      </c>
+      <c r="F68" s="13" t="n">
+        <f aca="false">F67*F65</f>
+        <v>840</v>
+      </c>
+      <c r="G68" s="13" t="n">
+        <f aca="false">$F$91</f>
+        <v>1860</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="F69" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>165</v>
+      <c r="A69" s="12" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B70" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="B70" s="4" t="s">
+      <c r="C70" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J24/C$68)</f>
+        <v>0.468538461538462</v>
+      </c>
+      <c r="D70" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K24/D$68)</f>
+        <v>0.0413504464285714</v>
+      </c>
+      <c r="E70" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L24/E$68)</f>
+        <v>0.466482426303855</v>
+      </c>
+      <c r="F70" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M24/F$68)</f>
+        <v>0.0598511904761905</v>
+      </c>
+      <c r="G70" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K24/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L24/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M24/Pallet!F23))/$F$90)</f>
+        <v>0.567684063208617</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C71" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J25/C$68)</f>
+        <v>0.351403846153846</v>
+      </c>
+      <c r="D71" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K25/D$68)</f>
+        <v>0.0330803571428571</v>
+      </c>
+      <c r="E71" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L25/E$68)</f>
+        <v>0.373185941043084</v>
+      </c>
+      <c r="F71" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M25/F$68)</f>
+        <v>0.0478809523809524</v>
+      </c>
+      <c r="G71" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K25/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L25/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M25/Pallet!F23))/$F$90)</f>
+        <v>0.454147250566894</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C72" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J26/C$68)</f>
+        <v>0.312358974358974</v>
+      </c>
+      <c r="D72" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K26/D$68)</f>
+        <v>0.0351478794642857</v>
+      </c>
+      <c r="E72" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L26/E$68)</f>
+        <v>0.396510062358277</v>
+      </c>
+      <c r="F72" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M26/F$68)</f>
+        <v>0.0508735119047619</v>
+      </c>
+      <c r="G72" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K26/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L26/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M26/Pallet!F23))/$F$90)</f>
+        <v>0.482531453727324</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C73" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J27/C$68)</f>
+        <v>0.292836538461538</v>
+      </c>
+      <c r="D73" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K27/D$68)</f>
+        <v>0.0351478794642857</v>
+      </c>
+      <c r="E73" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L27/E$68)</f>
+        <v>0.396510062358277</v>
+      </c>
+      <c r="F73" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M27/F$68)</f>
+        <v>0.0508735119047619</v>
+      </c>
+      <c r="G73" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K27/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L27/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M27/Pallet!F23))/$F$90)</f>
+        <v>0.482531453727324</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C74" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J28/C$68)</f>
+        <v>0.273314102564103</v>
+      </c>
+      <c r="D74" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K28/D$68)</f>
+        <v>0.0330803571428571</v>
+      </c>
+      <c r="E74" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L28/E$68)</f>
+        <v>0.373185941043084</v>
+      </c>
+      <c r="F74" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M28/F$68)</f>
+        <v>0.0478809523809524</v>
+      </c>
+      <c r="G74" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K28/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L28/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M28/Pallet!F23))/$F$90)</f>
+        <v>0.454147250566894</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C75" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J29/C$68)</f>
+        <v>0.273314102564103</v>
+      </c>
+      <c r="D75" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K29/D$68)</f>
+        <v>0.0310128348214286</v>
+      </c>
+      <c r="E75" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L29/E$68)</f>
+        <v>0.349861819727891</v>
+      </c>
+      <c r="F75" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M29/F$68)</f>
+        <v>0.0448883928571429</v>
+      </c>
+      <c r="G75" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K29/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L29/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M29/Pallet!F23))/$F$90)</f>
+        <v>0.425763047406463</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C76" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J30/C$68)</f>
+        <v>0.292836538461538</v>
+      </c>
+      <c r="D76" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K30/D$68)</f>
+        <v>0.0330803571428571</v>
+      </c>
+      <c r="E76" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L30/E$68)</f>
+        <v>0.373185941043084</v>
+      </c>
+      <c r="F76" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M30/F$68)</f>
+        <v>0.0478809523809524</v>
+      </c>
+      <c r="G76" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K30/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L30/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M30/Pallet!F23))/$F$90)</f>
+        <v>0.454147250566894</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C77" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J31/C$68)</f>
+        <v>0.292836538461538</v>
+      </c>
+      <c r="D77" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K31/D$68)</f>
+        <v>0.0330803571428571</v>
+      </c>
+      <c r="E77" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L31/E$68)</f>
+        <v>0.373185941043084</v>
+      </c>
+      <c r="F77" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M31/F$68)</f>
+        <v>0.0478809523809524</v>
+      </c>
+      <c r="G77" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K31/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L31/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M31/Pallet!F23))/$F$90)</f>
+        <v>0.454147250566894</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C78" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J32/C$68)</f>
+        <v>0.292836538461538</v>
+      </c>
+      <c r="D78" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K32/D$68)</f>
+        <v>0.0330803571428571</v>
+      </c>
+      <c r="E78" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L32/E$68)</f>
+        <v>0.373185941043084</v>
+      </c>
+      <c r="F78" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M32/F$68)</f>
+        <v>0.0478809523809524</v>
+      </c>
+      <c r="G78" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K32/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L32/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M32/Pallet!F23))/$F$90)</f>
+        <v>0.454147250566894</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C79" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J33/C$68)</f>
+        <v>0.292836538461538</v>
+      </c>
+      <c r="D79" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K33/D$68)</f>
+        <v>0.0310128348214286</v>
+      </c>
+      <c r="E79" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L33/E$68)</f>
+        <v>0.349861819727891</v>
+      </c>
+      <c r="F79" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M33/F$68)</f>
+        <v>0.0448883928571429</v>
+      </c>
+      <c r="G79" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K33/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L33/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M33/Pallet!F23))/$F$90)</f>
+        <v>0.425763047406463</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C80" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J34/C$68)</f>
+        <v>0.292836538461538</v>
+      </c>
+      <c r="D80" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K34/D$68)</f>
+        <v>0.0289453125</v>
+      </c>
+      <c r="E80" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L34/E$68)</f>
+        <v>0.326537698412698</v>
+      </c>
+      <c r="F80" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M34/F$68)</f>
+        <v>0.0418958333333333</v>
+      </c>
+      <c r="G80" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K34/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L34/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M34/Pallet!F23))/$F$90)</f>
+        <v>0.397378844246032</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C81" s="17" t="n">
+        <f aca="false">IF(C$68=0,0,Produccion!J35/C$68)</f>
+        <v>0.468538461538462</v>
+      </c>
+      <c r="D81" s="17" t="n">
+        <f aca="false">IF(D$68=0,0,Produccion!K35/D$68)</f>
+        <v>0.0454854910714286</v>
+      </c>
+      <c r="E81" s="17" t="n">
+        <f aca="false">IF(E$68=0,0,Produccion!L35/E$68)</f>
+        <v>0.51313066893424</v>
+      </c>
+      <c r="F81" s="17" t="n">
+        <f aca="false">IF(F$68=0,0,Produccion!M35/F$68)</f>
+        <v>0.0658363095238095</v>
+      </c>
+      <c r="G81" s="17" t="n">
+        <f aca="false">IF($F$90=0,0,(IF(Pallet!D23=0,0,Produccion!K35/Pallet!D23)+IF(Pallet!E23=0,0,Produccion!L35/Pallet!E23)+IF(Pallet!F23=0,0,Produccion!M35/Pallet!F23))/$F$90)</f>
+        <v>0.624452469529478</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C82" s="19" t="n">
+        <f aca="false">MAX(C70:C81)</f>
+        <v>0.468538461538462</v>
+      </c>
+      <c r="D82" s="19" t="n">
+        <f aca="false">MAX(D70:D81)</f>
+        <v>0.0454854910714286</v>
+      </c>
+      <c r="E82" s="19" t="n">
+        <f aca="false">MAX(E70:E81)</f>
+        <v>0.51313066893424</v>
+      </c>
+      <c r="F82" s="19" t="n">
+        <f aca="false">MAX(F70:F81)</f>
+        <v>0.0658363095238095</v>
+      </c>
+      <c r="G82" s="19" t="n">
+        <f aca="false">MAX(G70:G81)</f>
+        <v>0.624452469529478</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B83" s="4"/>
+      <c r="C83" s="20" t="str">
+        <f aca="false">IF(C82=0,"-",IF(C82&gt;=1,ROUNDUP(C82,0)&amp;" por semana",IF(INT(1/C82)=1,"1 por semana","1 cada "&amp;INT(1/C82)&amp;" semanas")))</f>
+        <v>1 cada 2 semanas</v>
+      </c>
+      <c r="D83" s="20" t="str">
+        <f aca="false">IF(D82=0,"-",IF(D82&gt;=1,ROUNDUP(D82,0)&amp;" por semana",IF(INT(1/D82)=1,"1 por semana","1 cada "&amp;INT(1/D82)&amp;" semanas")))</f>
+        <v>1 cada 21 semanas</v>
+      </c>
+      <c r="E83" s="20" t="str">
+        <f aca="false">IF(E82=0,"-",IF(E82&gt;=1,ROUNDUP(E82,0)&amp;" por semana",IF(INT(1/E82)=1,"1 por semana","1 cada "&amp;INT(1/E82)&amp;" semanas")))</f>
+        <v>1 por semana</v>
+      </c>
+      <c r="F83" s="20" t="str">
+        <f aca="false">IF(F82=0,"-",IF(F82&gt;=1,ROUNDUP(F82,0)&amp;" por semana",IF(INT(1/F82)=1,"1 por semana","1 cada "&amp;INT(1/F82)&amp;" semanas")))</f>
+        <v>1 cada 15 semanas</v>
+      </c>
+      <c r="G83" s="20" t="str">
+        <f aca="false">IF(G82=0,"-",IF(G82&gt;=1,ROUNDUP(G82,0)&amp;" por semana",IF(INT(1/G82)=1,"1 por semana","1 cada "&amp;INT(1/G82)&amp;" semanas")))</f>
+        <v>1 por semana</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C84" s="15" t="n">
+        <f aca="false">IF(C82=0,0,IF(C82&gt;=1,C82/ROUNDUP(C82,0),C82*INT(1/C82)))</f>
+        <v>0.937076923076923</v>
+      </c>
+      <c r="D84" s="15" t="n">
+        <f aca="false">IF(D82=0,0,IF(D82&gt;=1,D82/ROUNDUP(D82,0),D82*INT(1/D82)))</f>
+        <v>0.9551953125</v>
+      </c>
+      <c r="E84" s="15" t="n">
+        <f aca="false">IF(E82=0,0,IF(E82&gt;=1,E82/ROUNDUP(E82,0),E82*INT(1/E82)))</f>
+        <v>0.51313066893424</v>
+      </c>
+      <c r="F84" s="15" t="n">
+        <f aca="false">IF(F82=0,0,IF(F82&gt;=1,F82/ROUNDUP(F82,0),F82*INT(1/F82)))</f>
+        <v>0.987544642857143</v>
+      </c>
+      <c r="G84" s="15" t="n">
+        <f aca="false">IF(G82=0,0,IF(G82&gt;=1,G82/ROUNDUP(G82,0),G82*INT(1/G82)))</f>
+        <v>0.624452469529478</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C87" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D87" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E87" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C88" s="17" t="n">
+        <f aca="false">IF(Pallet!D23=0,0,Produccion!K36/Pallet!D23)</f>
+        <v>0.636796875</v>
+      </c>
+      <c r="D88" s="17" t="n">
+        <f aca="false">IF(Pallet!E23=0,0,Produccion!L36/Pallet!E23)</f>
+        <v>7.18382936507937</v>
+      </c>
+      <c r="E88" s="17" t="n">
+        <f aca="false">IF(Pallet!F23=0,0,Produccion!M36/Pallet!F23)</f>
+        <v>0.921708333333333</v>
+      </c>
+      <c r="F88" s="17" t="n">
+        <f aca="false">SUM(C88:E88)</f>
+        <v>8.7423345734127</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C89" s="15" t="n">
+        <f aca="false">IF($F88=0,0,C88/$F88)</f>
+        <v>0.0728405976289943</v>
+      </c>
+      <c r="D89" s="15" t="n">
+        <f aca="false">IF($F88=0,0,D88/$F88)</f>
+        <v>0.821728944912143</v>
+      </c>
+      <c r="E89" s="15" t="n">
+        <f aca="false">IF($F88=0,0,E88/$F88)</f>
+        <v>0.105430457458863</v>
+      </c>
+      <c r="F89" s="15" t="n">
+        <f aca="false">SUM(C89:E89)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C90" s="13" t="n">
+        <f aca="false">ROUND(SUM($C89:C89)*$F90,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D90" s="13" t="n">
+        <f aca="false">ROUND(SUM($C89:D89)*$F90,0)-ROUND(SUM($C89:C89)*$F90,0)</f>
+        <v>12</v>
+      </c>
+      <c r="E90" s="13" t="n">
+        <f aca="false">ROUND(SUM($C89:E89)*$F90,0)-ROUND(SUM($C89:D89)*$F90,0)</f>
+        <v>1</v>
+      </c>
+      <c r="F90" s="13" t="n">
+        <f aca="false">IF(F88=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/(C89*Pallet!D24+D89*Pallet!E24+E89*Pallet!F24))))</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B91" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C70" s="16" t="n">
+      <c r="C91" s="16" t="n">
+        <f aca="false">C90*Pallet!D23</f>
+        <v>288</v>
+      </c>
+      <c r="D91" s="16" t="n">
+        <f aca="false">D90*Pallet!E23</f>
+        <v>1512</v>
+      </c>
+      <c r="E91" s="16" t="n">
+        <f aca="false">E90*Pallet!F23</f>
+        <v>60</v>
+      </c>
+      <c r="F91" s="16" t="n">
+        <f aca="false">SUM(C91:E91)</f>
+        <v>1860</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C92" s="16" t="n">
+        <f aca="false">C90*Pallet!D24</f>
+        <v>464.24</v>
+      </c>
+      <c r="D92" s="16" t="n">
+        <f aca="false">D90*Pallet!E24</f>
+        <v>4652.16</v>
+      </c>
+      <c r="E92" s="16" t="n">
+        <f aca="false">E90*Pallet!F24</f>
+        <v>365.6</v>
+      </c>
+      <c r="F92" s="16" t="n">
+        <f aca="false">SUM(C92:E92)</f>
+        <v>5482</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="2"/>
+      <c r="B96" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="D96" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C97" s="16" t="n">
         <f aca="false">Pallet!G23</f>
         <v>24</v>
       </c>
-      <c r="D70" s="16" t="n">
+      <c r="D97" s="16" t="n">
         <f aca="false">Pallet!H23</f>
         <v>9</v>
       </c>
-      <c r="E70" s="16" t="n">
+      <c r="E97" s="16" t="n">
         <f aca="false">Pallet!I23</f>
         <v>6</v>
       </c>
-      <c r="F70" s="16" t="n">
+      <c r="F97" s="16" t="n">
         <f aca="false">Pallet!J23</f>
         <v>6</v>
       </c>
-      <c r="G70" s="16" t="n">
-        <f aca="false">IF((IF(Pallet!G23=0,0,Produccion!N$13/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O$13/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P$13/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q$13/Pallet!J23))=0,0,(Produccion!N$13+Produccion!O$13+Produccion!P$13+Produccion!Q$13)/(IF(Pallet!G23=0,0,Produccion!N$13/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O$13/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P$13/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q$13/Pallet!J23)))</f>
-        <v>9.53922174181593</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="B71" s="4" t="s">
+      <c r="G97" s="18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B98" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C71" s="16" t="n">
+      <c r="C98" s="16" t="n">
         <f aca="false">Pallet!G24</f>
         <v>418.88</v>
       </c>
-      <c r="D71" s="16" t="n">
+      <c r="D98" s="16" t="n">
         <f aca="false">Pallet!H24</f>
         <v>245.9</v>
       </c>
-      <c r="E71" s="16" t="n">
+      <c r="E98" s="16" t="n">
         <f aca="false">Pallet!I24</f>
         <v>317.37057704</v>
       </c>
-      <c r="F71" s="16" t="n">
+      <c r="F98" s="16" t="n">
         <f aca="false">Pallet!J24</f>
         <v>377.27790434</v>
       </c>
-      <c r="G71" s="16" t="n">
-        <f aca="false">IF((IF(Pallet!G23=0,0,Produccion!N$13/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O$13/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P$13/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q$13/Pallet!J23))=0,0,(Produccion!N$13/Pallet!G23*Pallet!G24+Produccion!O$13/Pallet!H23*Pallet!H24+Produccion!P$13/Pallet!I23*Pallet!I24+Produccion!Q$13/Pallet!J23*Pallet!J24)/(IF(Pallet!G23=0,0,Produccion!N$13/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O$13/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P$13/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q$13/Pallet!J23)))</f>
-        <v>293.340859399481</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="B72" s="4" t="s">
+      <c r="G98" s="18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="B99" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C72" s="13" t="n">
-        <f aca="false">IF(C71=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/C71)))</f>
+      <c r="C99" s="13" t="n">
+        <f aca="false">IF(C98=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/C98)))</f>
         <v>14</v>
       </c>
-      <c r="D72" s="13" t="n">
-        <f aca="false">IF(D71=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/D71)))</f>
+      <c r="D99" s="13" t="n">
+        <f aca="false">IF(D98=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/D98)))</f>
         <v>14</v>
       </c>
-      <c r="E72" s="13" t="n">
-        <f aca="false">IF(E71=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/E71)))</f>
+      <c r="E99" s="13" t="n">
+        <f aca="false">IF(E98=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/E98)))</f>
         <v>14</v>
       </c>
-      <c r="F72" s="13" t="n">
-        <f aca="false">IF(F71=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/F71)))</f>
+      <c r="F99" s="13" t="n">
+        <f aca="false">IF(F98=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/F98)))</f>
         <v>14</v>
       </c>
-      <c r="G72" s="13" t="n">
-        <f aca="false">IF(G71=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/G71)))</f>
+      <c r="G99" s="13" t="n">
+        <f aca="false">$G$122</f>
         <v>14</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="12" t="s">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C100" s="13" t="n">
+        <f aca="false">C99*C97</f>
+        <v>336</v>
+      </c>
+      <c r="D100" s="13" t="n">
+        <f aca="false">D99*D97</f>
+        <v>126</v>
+      </c>
+      <c r="E100" s="13" t="n">
+        <f aca="false">E99*E97</f>
+        <v>84</v>
+      </c>
+      <c r="F100" s="13" t="n">
+        <f aca="false">F99*F97</f>
+        <v>84</v>
+      </c>
+      <c r="G100" s="13" t="n">
+        <f aca="false">$G$123</f>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="12" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C102" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N24/C$100)</f>
+        <v>0.0203645833333333</v>
+      </c>
+      <c r="D102" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O24/D$100)</f>
+        <v>0.119404761904762</v>
+      </c>
+      <c r="E102" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P24/E$100)</f>
+        <v>0.0392113095238095</v>
+      </c>
+      <c r="F102" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q24/F$100)</f>
+        <v>0.0258035714285714</v>
+      </c>
+      <c r="G102" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N24/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O24/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P24/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q24/Pallet!J23))/$G$122)</f>
+        <v>0.204784226190476</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C103" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N25/C$100)</f>
+        <v>0.01796875</v>
+      </c>
+      <c r="D103" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O25/D$100)</f>
+        <v>0.105357142857143</v>
+      </c>
+      <c r="E103" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P25/E$100)</f>
+        <v>0.0345982142857143</v>
+      </c>
+      <c r="F103" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q25/F$100)</f>
+        <v>0.0227678571428571</v>
+      </c>
+      <c r="G103" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N25/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O25/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P25/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q25/Pallet!J23))/$G$122)</f>
+        <v>0.180691964285714</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C104" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N26/C$100)</f>
+        <v>0.0215625</v>
+      </c>
+      <c r="D104" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O26/D$100)</f>
+        <v>0.126428571428571</v>
+      </c>
+      <c r="E104" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P26/E$100)</f>
+        <v>0.0415178571428571</v>
+      </c>
+      <c r="F104" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q26/F$100)</f>
+        <v>0.0273214285714286</v>
+      </c>
+      <c r="G104" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N26/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O26/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P26/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q26/Pallet!J23))/$G$122)</f>
+        <v>0.216830357142857</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C105" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N27/C$100)</f>
+        <v>0.0215625</v>
+      </c>
+      <c r="D105" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O27/D$100)</f>
+        <v>0.126428571428571</v>
+      </c>
+      <c r="E105" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P27/E$100)</f>
+        <v>0.0415178571428571</v>
+      </c>
+      <c r="F105" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q27/F$100)</f>
+        <v>0.0273214285714286</v>
+      </c>
+      <c r="G105" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N27/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O27/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P27/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q27/Pallet!J23))/$G$122)</f>
+        <v>0.216830357142857</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C106" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N28/C$100)</f>
+        <v>0.0215625</v>
+      </c>
+      <c r="D106" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O28/D$100)</f>
+        <v>0.126428571428571</v>
+      </c>
+      <c r="E106" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P28/E$100)</f>
+        <v>0.0415178571428571</v>
+      </c>
+      <c r="F106" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q28/F$100)</f>
+        <v>0.0273214285714286</v>
+      </c>
+      <c r="G106" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N28/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O28/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P28/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q28/Pallet!J23))/$G$122)</f>
+        <v>0.216830357142857</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C107" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N29/C$100)</f>
+        <v>0.0191666666666667</v>
+      </c>
+      <c r="D107" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O29/D$100)</f>
+        <v>0.112380952380952</v>
+      </c>
+      <c r="E107" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P29/E$100)</f>
+        <v>0.0369047619047619</v>
+      </c>
+      <c r="F107" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q29/F$100)</f>
+        <v>0.0242857142857143</v>
+      </c>
+      <c r="G107" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N29/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O29/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P29/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q29/Pallet!J23))/$G$122)</f>
+        <v>0.192738095238095</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C108" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N30/C$100)</f>
+        <v>0.0215625</v>
+      </c>
+      <c r="D108" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O30/D$100)</f>
+        <v>0.126428571428571</v>
+      </c>
+      <c r="E108" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P30/E$100)</f>
+        <v>0.0415178571428571</v>
+      </c>
+      <c r="F108" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q30/F$100)</f>
+        <v>0.0273214285714286</v>
+      </c>
+      <c r="G108" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N30/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O30/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P30/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q30/Pallet!J23))/$G$122)</f>
+        <v>0.216830357142857</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C109" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N31/C$100)</f>
+        <v>0.0215625</v>
+      </c>
+      <c r="D109" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O31/D$100)</f>
+        <v>0.126428571428571</v>
+      </c>
+      <c r="E109" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P31/E$100)</f>
+        <v>0.0415178571428571</v>
+      </c>
+      <c r="F109" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q31/F$100)</f>
+        <v>0.0273214285714286</v>
+      </c>
+      <c r="G109" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N31/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O31/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P31/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q31/Pallet!J23))/$G$122)</f>
+        <v>0.216830357142857</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C110" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N32/C$100)</f>
+        <v>0.0203645833333333</v>
+      </c>
+      <c r="D110" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O32/D$100)</f>
+        <v>0.119404761904762</v>
+      </c>
+      <c r="E110" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P32/E$100)</f>
+        <v>0.0392113095238095</v>
+      </c>
+      <c r="F110" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q32/F$100)</f>
+        <v>0.0258035714285714</v>
+      </c>
+      <c r="G110" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N32/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O32/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P32/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q32/Pallet!J23))/$G$122)</f>
+        <v>0.204784226190476</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C111" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N33/C$100)</f>
+        <v>0.01796875</v>
+      </c>
+      <c r="D111" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O33/D$100)</f>
+        <v>0.105357142857143</v>
+      </c>
+      <c r="E111" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P33/E$100)</f>
+        <v>0.0345982142857143</v>
+      </c>
+      <c r="F111" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q33/F$100)</f>
+        <v>0.0227678571428571</v>
+      </c>
+      <c r="G111" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N33/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O33/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P33/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q33/Pallet!J23))/$G$122)</f>
+        <v>0.180691964285714</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C112" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N34/C$100)</f>
+        <v>0.0167708333333333</v>
+      </c>
+      <c r="D112" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O34/D$100)</f>
+        <v>0.0983333333333333</v>
+      </c>
+      <c r="E112" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P34/E$100)</f>
+        <v>0.0322916666666667</v>
+      </c>
+      <c r="F112" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q34/F$100)</f>
+        <v>0.02125</v>
+      </c>
+      <c r="G112" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N34/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O34/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P34/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q34/Pallet!J23))/$G$122)</f>
+        <v>0.168645833333333</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C113" s="17" t="n">
+        <f aca="false">IF(C$100=0,0,Produccion!N35/C$100)</f>
+        <v>0.0191666666666667</v>
+      </c>
+      <c r="D113" s="17" t="n">
+        <f aca="false">IF(D$100=0,0,Produccion!O35/D$100)</f>
+        <v>0.112380952380952</v>
+      </c>
+      <c r="E113" s="17" t="n">
+        <f aca="false">IF(E$100=0,0,Produccion!P35/E$100)</f>
+        <v>0.0369047619047619</v>
+      </c>
+      <c r="F113" s="17" t="n">
+        <f aca="false">IF(F$100=0,0,Produccion!Q35/F$100)</f>
+        <v>0.0242857142857143</v>
+      </c>
+      <c r="G113" s="17" t="n">
+        <f aca="false">IF($G$122=0,0,(IF(Pallet!G23=0,0,Produccion!N35/Pallet!G23)+IF(Pallet!H23=0,0,Produccion!O35/Pallet!H23)+IF(Pallet!I23=0,0,Produccion!P35/Pallet!I23)+IF(Pallet!J23=0,0,Produccion!Q35/Pallet!J23))/$G$122)</f>
+        <v>0.192738095238095</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="B73" s="4" t="s">
+      <c r="B114" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="C114" s="19" t="n">
+        <f aca="false">MAX(C102:C113)</f>
+        <v>0.0215625</v>
+      </c>
+      <c r="D114" s="19" t="n">
+        <f aca="false">MAX(D102:D113)</f>
+        <v>0.126428571428571</v>
+      </c>
+      <c r="E114" s="19" t="n">
+        <f aca="false">MAX(E102:E113)</f>
+        <v>0.0415178571428571</v>
+      </c>
+      <c r="F114" s="19" t="n">
+        <f aca="false">MAX(F102:F113)</f>
+        <v>0.0273214285714286</v>
+      </c>
+      <c r="G114" s="19" t="n">
+        <f aca="false">MAX(G102:G113)</f>
+        <v>0.216830357142857</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B115" s="4"/>
+      <c r="C115" s="20" t="str">
+        <f aca="false">IF(C114=0,"-",IF(C114&gt;=1,ROUNDUP(C114,0)&amp;" por semana",IF(INT(1/C114)=1,"1 por semana","1 cada "&amp;INT(1/C114)&amp;" semanas")))</f>
+        <v>1 cada 46 semanas</v>
+      </c>
+      <c r="D115" s="20" t="str">
+        <f aca="false">IF(D114=0,"-",IF(D114&gt;=1,ROUNDUP(D114,0)&amp;" por semana",IF(INT(1/D114)=1,"1 por semana","1 cada "&amp;INT(1/D114)&amp;" semanas")))</f>
+        <v>1 cada 7 semanas</v>
+      </c>
+      <c r="E115" s="20" t="str">
+        <f aca="false">IF(E114=0,"-",IF(E114&gt;=1,ROUNDUP(E114,0)&amp;" por semana",IF(INT(1/E114)=1,"1 por semana","1 cada "&amp;INT(1/E114)&amp;" semanas")))</f>
+        <v>1 cada 24 semanas</v>
+      </c>
+      <c r="F115" s="20" t="str">
+        <f aca="false">IF(F114=0,"-",IF(F114&gt;=1,ROUNDUP(F114,0)&amp;" por semana",IF(INT(1/F114)=1,"1 por semana","1 cada "&amp;INT(1/F114)&amp;" semanas")))</f>
+        <v>1 cada 36 semanas</v>
+      </c>
+      <c r="G115" s="20" t="str">
+        <f aca="false">IF(G114=0,"-",IF(G114&gt;=1,ROUNDUP(G114,0)&amp;" por semana",IF(INT(1/G114)=1,"1 por semana","1 cada "&amp;INT(1/G114)&amp;" semanas")))</f>
+        <v>1 cada 4 semanas</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C116" s="15" t="n">
+        <f aca="false">IF(C114=0,0,IF(C114&gt;=1,C114/ROUNDUP(C114,0),C114*INT(1/C114)))</f>
+        <v>0.991875</v>
+      </c>
+      <c r="D116" s="15" t="n">
+        <f aca="false">IF(D114=0,0,IF(D114&gt;=1,D114/ROUNDUP(D114,0),D114*INT(1/D114)))</f>
+        <v>0.885</v>
+      </c>
+      <c r="E116" s="15" t="n">
+        <f aca="false">IF(E114=0,0,IF(E114&gt;=1,E114/ROUNDUP(E114,0),E114*INT(1/E114)))</f>
+        <v>0.996428571428571</v>
+      </c>
+      <c r="F116" s="15" t="n">
+        <f aca="false">IF(F114=0,0,IF(F114&gt;=1,F114/ROUNDUP(F114,0),F114*INT(1/F114)))</f>
+        <v>0.983571428571429</v>
+      </c>
+      <c r="G116" s="15" t="n">
+        <f aca="false">IF(G114=0,0,IF(G114&gt;=1,G114/ROUNDUP(G114,0),G114*INT(1/G114)))</f>
+        <v>0.867321428571429</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="2"/>
+      <c r="B119" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C119" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G119" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C120" s="17" t="n">
+        <f aca="false">IF(Pallet!G23=0,0,Produccion!N36/Pallet!G23)</f>
+        <v>0.301875</v>
+      </c>
+      <c r="D120" s="17" t="n">
+        <f aca="false">IF(Pallet!H23=0,0,Produccion!O36/Pallet!H23)</f>
+        <v>1.77</v>
+      </c>
+      <c r="E120" s="17" t="n">
+        <f aca="false">IF(Pallet!I23=0,0,Produccion!P36/Pallet!I23)</f>
+        <v>0.58125</v>
+      </c>
+      <c r="F120" s="17" t="n">
+        <f aca="false">IF(Pallet!J23=0,0,Produccion!Q36/Pallet!J23)</f>
+        <v>0.3825</v>
+      </c>
+      <c r="G120" s="17" t="n">
+        <f aca="false">SUM(C120:F120)</f>
+        <v>3.035625</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="C121" s="15" t="n">
+        <f aca="false">IF($G120=0,0,C120/$G120)</f>
+        <v>0.099444101297097</v>
+      </c>
+      <c r="D121" s="15" t="n">
+        <f aca="false">IF($G120=0,0,D120/$G120)</f>
+        <v>0.58307597282273</v>
+      </c>
+      <c r="E121" s="15" t="n">
+        <f aca="false">IF($G120=0,0,E120/$G120)</f>
+        <v>0.19147621988882</v>
+      </c>
+      <c r="F121" s="15" t="n">
+        <f aca="false">IF($G120=0,0,F120/$G120)</f>
+        <v>0.126003705991353</v>
+      </c>
+      <c r="G121" s="15" t="n">
+        <f aca="false">SUM(C121:F121)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="C122" s="13" t="n">
+        <f aca="false">ROUND(SUM($C121:C121)*$G122,0)</f>
+        <v>1</v>
+      </c>
+      <c r="D122" s="13" t="n">
+        <f aca="false">ROUND(SUM($C121:D121)*$G122,0)-ROUND(SUM($C121:C121)*$G122,0)</f>
+        <v>9</v>
+      </c>
+      <c r="E122" s="13" t="n">
+        <f aca="false">ROUND(SUM($C121:E121)*$G122,0)-ROUND(SUM($C121:D121)*$G122,0)</f>
+        <v>2</v>
+      </c>
+      <c r="F122" s="13" t="n">
+        <f aca="false">ROUND(SUM($C121:F121)*$G122,0)-ROUND(SUM($C121:E121)*$G122,0)</f>
+        <v>2</v>
+      </c>
+      <c r="G122" s="13" t="n">
+        <f aca="false">IF(G120=0,0,MIN(Camion!$C$5,INT(Datos!$C$42/(C121*Pallet!G24+D121*Pallet!H24+E121*Pallet!I24+F121*Pallet!J24))))</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B123" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C73" s="13" t="n">
-        <f aca="false">C72*C70</f>
-        <v>336</v>
-      </c>
-      <c r="D73" s="13" t="n">
-        <f aca="false">D72*D70</f>
-        <v>126</v>
-      </c>
-      <c r="E73" s="13" t="n">
-        <f aca="false">E72*E70</f>
-        <v>84</v>
-      </c>
-      <c r="F73" s="13" t="n">
-        <f aca="false">F72*F70</f>
-        <v>84</v>
-      </c>
-      <c r="G73" s="13" t="n">
-        <f aca="false">G72*G70</f>
-        <v>133.549104385423</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="12" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B75" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C75" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N24/C$73)</f>
-        <v>0.0203645833333333</v>
-      </c>
-      <c r="D75" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O24/D$73)</f>
-        <v>0.119404761904762</v>
-      </c>
-      <c r="E75" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P24/E$73)</f>
-        <v>0.0392113095238095</v>
-      </c>
-      <c r="F75" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q24/F$73)</f>
-        <v>0.0258035714285714</v>
-      </c>
-      <c r="G75" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U24/G$73)</f>
-        <v>0.204784226190476</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C76" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N25/C$73)</f>
-        <v>0.01796875</v>
-      </c>
-      <c r="D76" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O25/D$73)</f>
-        <v>0.105357142857143</v>
-      </c>
-      <c r="E76" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P25/E$73)</f>
-        <v>0.0345982142857143</v>
-      </c>
-      <c r="F76" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q25/F$73)</f>
-        <v>0.0227678571428571</v>
-      </c>
-      <c r="G76" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U25/G$73)</f>
-        <v>0.180691964285714</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B77" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C77" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N26/C$73)</f>
-        <v>0.0215625</v>
-      </c>
-      <c r="D77" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O26/D$73)</f>
-        <v>0.126428571428571</v>
-      </c>
-      <c r="E77" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P26/E$73)</f>
-        <v>0.0415178571428571</v>
-      </c>
-      <c r="F77" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q26/F$73)</f>
-        <v>0.0273214285714286</v>
-      </c>
-      <c r="G77" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U26/G$73)</f>
-        <v>0.216830357142857</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C78" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N27/C$73)</f>
-        <v>0.0215625</v>
-      </c>
-      <c r="D78" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O27/D$73)</f>
-        <v>0.126428571428571</v>
-      </c>
-      <c r="E78" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P27/E$73)</f>
-        <v>0.0415178571428571</v>
-      </c>
-      <c r="F78" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q27/F$73)</f>
-        <v>0.0273214285714286</v>
-      </c>
-      <c r="G78" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U27/G$73)</f>
-        <v>0.216830357142857</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C79" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N28/C$73)</f>
-        <v>0.0215625</v>
-      </c>
-      <c r="D79" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O28/D$73)</f>
-        <v>0.126428571428571</v>
-      </c>
-      <c r="E79" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P28/E$73)</f>
-        <v>0.0415178571428571</v>
-      </c>
-      <c r="F79" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q28/F$73)</f>
-        <v>0.0273214285714286</v>
-      </c>
-      <c r="G79" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U28/G$73)</f>
-        <v>0.216830357142857</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C80" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N29/C$73)</f>
-        <v>0.0191666666666667</v>
-      </c>
-      <c r="D80" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O29/D$73)</f>
-        <v>0.112380952380952</v>
-      </c>
-      <c r="E80" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P29/E$73)</f>
-        <v>0.0369047619047619</v>
-      </c>
-      <c r="F80" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q29/F$73)</f>
-        <v>0.0242857142857143</v>
-      </c>
-      <c r="G80" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U29/G$73)</f>
-        <v>0.192738095238095</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C81" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N30/C$73)</f>
-        <v>0.0215625</v>
-      </c>
-      <c r="D81" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O30/D$73)</f>
-        <v>0.126428571428571</v>
-      </c>
-      <c r="E81" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P30/E$73)</f>
-        <v>0.0415178571428571</v>
-      </c>
-      <c r="F81" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q30/F$73)</f>
-        <v>0.0273214285714286</v>
-      </c>
-      <c r="G81" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U30/G$73)</f>
-        <v>0.216830357142857</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B82" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C82" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N31/C$73)</f>
-        <v>0.0215625</v>
-      </c>
-      <c r="D82" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O31/D$73)</f>
-        <v>0.126428571428571</v>
-      </c>
-      <c r="E82" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P31/E$73)</f>
-        <v>0.0415178571428571</v>
-      </c>
-      <c r="F82" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q31/F$73)</f>
-        <v>0.0273214285714286</v>
-      </c>
-      <c r="G82" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U31/G$73)</f>
-        <v>0.216830357142857</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C83" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N32/C$73)</f>
-        <v>0.0203645833333333</v>
-      </c>
-      <c r="D83" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O32/D$73)</f>
-        <v>0.119404761904762</v>
-      </c>
-      <c r="E83" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P32/E$73)</f>
-        <v>0.0392113095238095</v>
-      </c>
-      <c r="F83" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q32/F$73)</f>
-        <v>0.0258035714285714</v>
-      </c>
-      <c r="G83" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U32/G$73)</f>
-        <v>0.204784226190476</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C84" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N33/C$73)</f>
-        <v>0.01796875</v>
-      </c>
-      <c r="D84" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O33/D$73)</f>
-        <v>0.105357142857143</v>
-      </c>
-      <c r="E84" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P33/E$73)</f>
-        <v>0.0345982142857143</v>
-      </c>
-      <c r="F84" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q33/F$73)</f>
-        <v>0.0227678571428571</v>
-      </c>
-      <c r="G84" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U33/G$73)</f>
-        <v>0.180691964285714</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C85" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N34/C$73)</f>
-        <v>0.0167708333333333</v>
-      </c>
-      <c r="D85" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O34/D$73)</f>
-        <v>0.0983333333333333</v>
-      </c>
-      <c r="E85" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P34/E$73)</f>
-        <v>0.0322916666666667</v>
-      </c>
-      <c r="F85" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q34/F$73)</f>
-        <v>0.02125</v>
-      </c>
-      <c r="G85" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U34/G$73)</f>
-        <v>0.168645833333333</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B86" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C86" s="17" t="n">
-        <f aca="false">IF(C$73=0,0,Produccion!N35/C$73)</f>
-        <v>0.0191666666666667</v>
-      </c>
-      <c r="D86" s="17" t="n">
-        <f aca="false">IF(D$73=0,0,Produccion!O35/D$73)</f>
-        <v>0.112380952380952</v>
-      </c>
-      <c r="E86" s="17" t="n">
-        <f aca="false">IF(E$73=0,0,Produccion!P35/E$73)</f>
-        <v>0.0369047619047619</v>
-      </c>
-      <c r="F86" s="17" t="n">
-        <f aca="false">IF(F$73=0,0,Produccion!Q35/F$73)</f>
-        <v>0.0242857142857143</v>
-      </c>
-      <c r="G86" s="17" t="n">
-        <f aca="false">IF(G$73=0,0,Produccion!U35/G$73)</f>
-        <v>0.192738095238095</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="B87" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C87" s="18" t="n">
-        <f aca="false">MAX(C75:C86)</f>
-        <v>0.0215625</v>
-      </c>
-      <c r="D87" s="18" t="n">
-        <f aca="false">MAX(D75:D86)</f>
-        <v>0.126428571428571</v>
-      </c>
-      <c r="E87" s="18" t="n">
-        <f aca="false">MAX(E75:E86)</f>
-        <v>0.0415178571428571</v>
-      </c>
-      <c r="F87" s="18" t="n">
-        <f aca="false">MAX(F75:F86)</f>
-        <v>0.0273214285714286</v>
-      </c>
-      <c r="G87" s="18" t="n">
-        <f aca="false">MAX(G75:G86)</f>
-        <v>0.216830357142857</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="B88" s="4"/>
-      <c r="C88" s="19" t="str">
-        <f aca="false">IF(C87=0,"-",IF(C87&gt;=1,ROUNDUP(C87,0)&amp;" por semana",IF(INT(1/C87)=1,"1 por semana","1 cada "&amp;INT(1/C87)&amp;" semanas")))</f>
-        <v>1 cada 46 semanas</v>
-      </c>
-      <c r="D88" s="19" t="str">
-        <f aca="false">IF(D87=0,"-",IF(D87&gt;=1,ROUNDUP(D87,0)&amp;" por semana",IF(INT(1/D87)=1,"1 por semana","1 cada "&amp;INT(1/D87)&amp;" semanas")))</f>
-        <v>1 cada 7 semanas</v>
-      </c>
-      <c r="E88" s="19" t="str">
-        <f aca="false">IF(E87=0,"-",IF(E87&gt;=1,ROUNDUP(E87,0)&amp;" por semana",IF(INT(1/E87)=1,"1 por semana","1 cada "&amp;INT(1/E87)&amp;" semanas")))</f>
-        <v>1 cada 24 semanas</v>
-      </c>
-      <c r="F88" s="19" t="str">
-        <f aca="false">IF(F87=0,"-",IF(F87&gt;=1,ROUNDUP(F87,0)&amp;" por semana",IF(INT(1/F87)=1,"1 por semana","1 cada "&amp;INT(1/F87)&amp;" semanas")))</f>
-        <v>1 cada 36 semanas</v>
-      </c>
-      <c r="G88" s="19" t="str">
-        <f aca="false">IF(G87=0,"-",IF(G87&gt;=1,ROUNDUP(G87,0)&amp;" por semana",IF(INT(1/G87)=1,"1 por semana","1 cada "&amp;INT(1/G87)&amp;" semanas")))</f>
-        <v>1 cada 4 semanas</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B89" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="C89" s="15" t="n">
-        <f aca="false">IF(C87=0,0,IF(C87&gt;=1,C87/ROUNDUP(C87,0),C87*INT(1/C87)))</f>
-        <v>0.991875</v>
-      </c>
-      <c r="D89" s="15" t="n">
-        <f aca="false">IF(D87=0,0,IF(D87&gt;=1,D87/ROUNDUP(D87,0),D87*INT(1/D87)))</f>
-        <v>0.885</v>
-      </c>
-      <c r="E89" s="15" t="n">
-        <f aca="false">IF(E87=0,0,IF(E87&gt;=1,E87/ROUNDUP(E87,0),E87*INT(1/E87)))</f>
-        <v>0.996428571428571</v>
-      </c>
-      <c r="F89" s="15" t="n">
-        <f aca="false">IF(F87=0,0,IF(F87&gt;=1,F87/ROUNDUP(F87,0),F87*INT(1/F87)))</f>
-        <v>0.983571428571429</v>
-      </c>
-      <c r="G89" s="15" t="n">
-        <f aca="false">IF(G87=0,0,IF(G87&gt;=1,G87/ROUNDUP(G87,0),G87*INT(1/G87)))</f>
-        <v>0.867321428571429</v>
+      <c r="C123" s="16" t="n">
+        <f aca="false">C122*Pallet!G23</f>
+        <v>24</v>
+      </c>
+      <c r="D123" s="16" t="n">
+        <f aca="false">D122*Pallet!H23</f>
+        <v>81</v>
+      </c>
+      <c r="E123" s="16" t="n">
+        <f aca="false">E122*Pallet!I23</f>
+        <v>12</v>
+      </c>
+      <c r="F123" s="16" t="n">
+        <f aca="false">F122*Pallet!J23</f>
+        <v>12</v>
+      </c>
+      <c r="G123" s="16" t="n">
+        <f aca="false">SUM(C123:F123)</f>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C124" s="16" t="n">
+        <f aca="false">C122*Pallet!G24</f>
+        <v>418.88</v>
+      </c>
+      <c r="D124" s="16" t="n">
+        <f aca="false">D122*Pallet!H24</f>
+        <v>2213.1</v>
+      </c>
+      <c r="E124" s="16" t="n">
+        <f aca="false">E122*Pallet!I24</f>
+        <v>634.74115408</v>
+      </c>
+      <c r="F124" s="16" t="n">
+        <f aca="false">F122*Pallet!J24</f>
+        <v>754.55580868</v>
+      </c>
+      <c r="G124" s="16" t="n">
+        <f aca="false">SUM(C124:F124)</f>
+        <v>4021.27696276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Palletizado: recargas de la planta industrial con sustitutos
Hojas Recargas y Recargas_camion: recargas de la planta industrial
(61,5 %), recargados + sustitutos como máximo, jaulas tipo A, tipo B y
pallets de rodantes del Word de recargas, y viajes del Iveco de 2 t con
el control del peso de un viaje lleno.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/palletizado_PT.xlsx
+++ b/salida/palletizado_PT.xlsx
@@ -13,6 +13,8 @@
     <sheet name="Pallet" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Camion" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Escenarios" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Recargas" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Recargas_camion" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="268">
   <si>
     <t xml:space="preserve">General</t>
   </si>
@@ -597,6 +599,237 @@
   </si>
   <si>
     <t xml:space="preserve">Cilindros de rodantes (sider)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargas anuales (Proyecciones 5, hoja Indexado Dim Técnico, filas 27 a 43)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 1 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 2,5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 10 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua 10 l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFFF 10 l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AFFF 50 l s/ruedas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC 5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales K 6 l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO₂ 2 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CO₂ 5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HCFC/HFC 5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clase D 9 l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 25 kg s/ruedas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 50 kg s/ruedas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 70 kg s/ruedas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABC 100 kg s/ruedas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta industrial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: zonas de la planta industrial (CABA Sur, PBA Sur, PBA Oeste e Interior), Indexado Dim Técnico filas 61 a 74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas metálicas palletizables de 1.200 × 1.000 (Word Proceso de recargas, Recepción y registro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U por jaula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A 1 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo A: 1 nivel, 8 × 9 celdas de 100 × 140 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B 2,5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo B multiformato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B 5 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B 10 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R 25 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pallet de rodantes: carros por 1.200 × 1.000 (huella de Datos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R 50 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R 70 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R 100 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datos de la recarga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sustitutos por extintor retirado (máximo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máximo: uno por extintor (IRAM 3517-2 9.4.5); la reserva del cliente cubre 6,5 % (Reservas y Sustitutos, fila 33)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tara de la jaula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio: base de acero 1.200 × 1.000 de 22 a 37,5 kg (fltgrupa.pl, hellopro.fr) + reja y varillas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Días hábiles por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">días</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lunes a viernes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta industrial: recargados + sustitutos por semana del año elegido (máximo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargas año (todas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta ind. por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso u. (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sustituto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sust. por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas sust.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kg por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clase sust.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuentes: formato, Word (ABC) y por tamaño el resto (criterio); peso, FLAMA_BOM hoja Resumen (peso de catálogo); sustituto, Reservas y Sustitutos filas 54 a 65.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camión de recargas: Iveco cabina simple con baranda rebatible (Word Proceso de recargas, Recepción y registro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas tipo A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas tipo B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pallets rodantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacidad por viaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo recargados por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargados + sustitutos por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viajes por semana: solo recargados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viajes por semana: con sustitutos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIAJES POR SEMANA (con sustitutos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viajes por día hábil (con sustitutos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camiones para 1 viaje por día</t>
+  </si>
+  <si>
+    <t xml:space="preserve">camiones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limita</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso de 9 jaulas A llenas de 1 kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso de un viaje lleno (9 A de 1 kg, 8 B de 5 kg, 2 pallets de 50 kg y jaulas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Entra en la carga útil?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente de la capacidad: 9 jaulas tipo A, 8 tipo B, 2 pallets de rodantes y unas 2 t de carga útil, con un pico de 1,2 t (Word Proceso de recargas, Recepción y registro).</t>
   </si>
 </sst>
 </file>
@@ -741,7 +974,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -835,6 +1068,18 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8323,4 +8568,2248 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:M60"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="2" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>2029</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>2030</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>2031</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>2032</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>2033</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>2034</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>3477.4821</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>16970.5856</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>30546.0895</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>56048.3111</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>84270.2261</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>117407.8231</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>147610.6356</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>171404.3607</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>183690.566</v>
+      </c>
+      <c r="K3" s="6" t="n">
+        <v>196282.6907</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>329.9967</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>1287.414</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>2947.1692</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>5426.0433</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>7850.8758</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>10423.9436</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>12809.8957</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>14263.0683</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>15432.8698</v>
+      </c>
+      <c r="K4" s="6" t="n">
+        <v>16620.7612</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1950.3941</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>7852.6185</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>17775.857</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>33605.5684</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>48407.5719</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>64323.0428</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>78721.1004</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>87237.2124</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>94103.6676</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>101095.1762</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>118.3436</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>437.7166</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>1024.9748</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1960.4099</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>2844.9768</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>3810.3906</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>4663.6781</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>5164.5146</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>5571.5443</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>5985.9509</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>159.3087</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>643.4235</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>1474.3627</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>2766.4512</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>3991.4652</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>5335.7558</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>6538.9589</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>7269.8197</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>7855.4414</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>8450.8141</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>22.7584</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>161.3158</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>316.6073</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>527.3946</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>743.7889</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>962.8743</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>1194.9422</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>1351.6172</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>1477.5489</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>1604.4414</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>11.3792</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>83.2235</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>164.4638</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>281.3411</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>398.9025</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>514.5273</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>629.0655</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>711.178</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>773.411</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>836.3508</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>6.8275</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>47.0731</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>88.8897</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>159.5025</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>219.7962</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>291.8699</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>368.8442</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>408.409</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>445.7819</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>483.4792</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>81.9302</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>335.3989</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>746.5984</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1358.8998</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>1961.1255</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>2598.5414</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>3197.2635</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>3578.5395</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>3870.748</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>4167.5596</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>450.6161</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>1697.1815</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>3955.1969</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>7561.2603</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>10920.1448</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>14514.8852</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>17746.4993</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>19617.2055</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>21161.8063</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>22734.5017</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>125.1711</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>643.6304</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>1375.6267</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>2460.2843</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>3545.2577</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>4723.4618</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>5853.9052</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>6608.4599</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>7185.7084</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>7769.5771</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>18.2067</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>112.0751</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>230.854</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>400.7153</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>574.5078</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>754.3456</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>944.8488</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>1072.2347</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>1171.6958</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>1271.9411</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>6.8275</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>47.0731</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>88.8897</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>148.2792</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>205.2261</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>255.7651</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>328.4179</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>366.9081</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>401.6817</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>436.6868</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>17.6378</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>85.9878</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>186.8696</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>336.5836</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>484.1326</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>643.2204</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>792.4317</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>889.6777</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>965.3111</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>1041.9397</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>38.8031</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>189.1732</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>411.113</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>740.484</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>1065.0917</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>1415.0848</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>1743.3498</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>1957.291</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>2123.6844</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>2292.2673</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>8.4661</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>41.2742</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>89.6974</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>161.5601</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>232.3836</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>308.7458</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>380.3672</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>427.0453</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>463.3493</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>500.1311</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>5.6441</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>27.5161</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>59.7983</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>107.7068</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>154.9224</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>205.8305</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>253.5782</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>284.6969</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>308.8996</v>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>333.4207</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" s="14" t="n">
+        <v>0.616614</v>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>0.616547</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>0.616464</v>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>0.616363</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>0.616237</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>0.616086</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>0.615903</v>
+      </c>
+      <c r="I20" s="14" t="n">
+        <v>0.615684</v>
+      </c>
+      <c r="J20" s="14" t="n">
+        <v>0.615422</v>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>0.615111</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C29" s="16" t="n">
+        <f aca="false">MAX(INT(Datos!$C$8/Datos!$C$34)*INT(Datos!$C$9/Datos!$C$35),INT(Datos!$C$8/Datos!$C$35)*INT(Datos!$C$9/Datos!$C$34))</f>
+        <v>2</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C30" s="16" t="n">
+        <f aca="false">MAX(INT(Datos!$C$8/Datos!$D$34)*INT(Datos!$C$9/Datos!$D$35),INT(Datos!$C$8/Datos!$D$35)*INT(Datos!$C$9/Datos!$D$34))</f>
+        <v>2</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C31" s="16" t="n">
+        <f aca="false">MAX(INT(Datos!$C$8/Datos!$E$34)*INT(Datos!$C$9/Datos!$E$35),INT(Datos!$C$8/Datos!$E$35)*INT(Datos!$C$9/Datos!$E$34))</f>
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C32" s="16" t="n">
+        <f aca="false">MAX(INT(Datos!$C$8/Datos!$F$34)*INT(Datos!$C$9/Datos!$F$35),INT(Datos!$C$8/Datos!$F$35)*INT(Datos!$C$9/Datos!$F$34))</f>
+        <v>1</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="C36" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" s="16" t="n">
+        <f aca="false">INDEX($B$3:$K$3,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>196282.6907</v>
+      </c>
+      <c r="C42" s="16" t="n">
+        <f aca="false">B42*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>2515.32587831599</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>216</v>
+      </c>
+      <c r="E42" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D42,$A$25:$A$32,0))</f>
+        <v>72</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <f aca="false">IF(E42=0,0,C42/E42)</f>
+        <v>34.9350816432777</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H42" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="I42" s="16" t="n">
+        <f aca="false">C42*$C$36</f>
+        <v>2515.32587831599</v>
+      </c>
+      <c r="J42" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H42,$A$42:$A$58,0))=0,0,I42/INDEX($E$42:$E$58,MATCH($H42,$A$42:$A$58,0)))</f>
+        <v>104.805244929833</v>
+      </c>
+      <c r="K42" s="16" t="n">
+        <f aca="false">C42*G42+I42*INDEX($G$42:$G$58,MATCH($H42,$A$42:$A$58,0))+(F42+J42)*$C$37</f>
+        <v>34543.808728873</v>
+      </c>
+      <c r="L42" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D42,$A$25:$A$32,0))</f>
+        <v>A</v>
+      </c>
+      <c r="M42" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H42,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="B43" s="16" t="n">
+        <f aca="false">INDEX($B$4:$K$4,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>16620.7612</v>
+      </c>
+      <c r="C43" s="16" t="n">
+        <f aca="false">B43*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>212.991938385275</v>
+      </c>
+      <c r="D43" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="E43" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D43,$A$25:$A$32,0))</f>
+        <v>30</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <f aca="false">IF(E43=0,0,C43/E43)</f>
+        <v>7.09973127950917</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="H43" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="I43" s="16" t="n">
+        <f aca="false">C43*$C$36</f>
+        <v>212.991938385275</v>
+      </c>
+      <c r="J43" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H43,$A$42:$A$58,0))=0,0,I43/INDEX($E$42:$E$58,MATCH($H43,$A$42:$A$58,0)))</f>
+        <v>8.87466409938646</v>
+      </c>
+      <c r="K43" s="16" t="n">
+        <f aca="false">C43*G43+I43*INDEX($G$42:$G$58,MATCH($H43,$A$42:$A$58,0))+(F43+J43)*$C$37</f>
+        <v>3748.65811558084</v>
+      </c>
+      <c r="L43" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D43,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M43" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H43,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="B44" s="16" t="n">
+        <f aca="false">INDEX($B$5:$K$5,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>101095.1762</v>
+      </c>
+      <c r="C44" s="16" t="n">
+        <f aca="false">B44*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>1295.51572765746</v>
+      </c>
+      <c r="D44" s="25" t="s">
+        <v>222</v>
+      </c>
+      <c r="E44" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D44,$A$25:$A$32,0))</f>
+        <v>24</v>
+      </c>
+      <c r="F44" s="17" t="n">
+        <f aca="false">IF(E44=0,0,C44/E44)</f>
+        <v>53.9798219857276</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H44" s="26" t="s">
+        <v>195</v>
+      </c>
+      <c r="I44" s="16" t="n">
+        <f aca="false">C44*$C$36</f>
+        <v>1295.51572765746</v>
+      </c>
+      <c r="J44" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H44,$A$42:$A$58,0))=0,0,I44/INDEX($E$42:$E$58,MATCH($H44,$A$42:$A$58,0)))</f>
+        <v>53.9798219857276</v>
+      </c>
+      <c r="K44" s="16" t="n">
+        <f aca="false">C44*G44+I44*INDEX($G$42:$G$58,MATCH($H44,$A$42:$A$58,0))+(F44+J44)*$C$37</f>
+        <v>28501.3460084642</v>
+      </c>
+      <c r="L44" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D44,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M44" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H44,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B45" s="16" t="n">
+        <f aca="false">INDEX($B$6:$K$6,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>5985.9509</v>
+      </c>
+      <c r="C45" s="16" t="n">
+        <f aca="false">B45*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>76.7088384177063</v>
+      </c>
+      <c r="D45" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E45" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D45,$A$25:$A$32,0))</f>
+        <v>16</v>
+      </c>
+      <c r="F45" s="17" t="n">
+        <f aca="false">IF(E45=0,0,C45/E45)</f>
+        <v>4.79430240110664</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H45" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="I45" s="16" t="n">
+        <f aca="false">C45*$C$36</f>
+        <v>76.7088384177063</v>
+      </c>
+      <c r="J45" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H45,$A$42:$A$58,0))=0,0,I45/INDEX($E$42:$E$58,MATCH($H45,$A$42:$A$58,0)))</f>
+        <v>4.79430240110664</v>
+      </c>
+      <c r="K45" s="16" t="n">
+        <f aca="false">C45*G45+I45*INDEX($G$42:$G$58,MATCH($H45,$A$42:$A$58,0))+(F45+J45)*$C$37</f>
+        <v>3106.7079559171</v>
+      </c>
+      <c r="L45" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D45,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M45" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H45,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="B46" s="16" t="n">
+        <f aca="false">INDEX($B$7:$K$7,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>8450.8141</v>
+      </c>
+      <c r="C46" s="16" t="n">
+        <f aca="false">B46*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>108.295598163856</v>
+      </c>
+      <c r="D46" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E46" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D46,$A$25:$A$32,0))</f>
+        <v>16</v>
+      </c>
+      <c r="F46" s="17" t="n">
+        <f aca="false">IF(E46=0,0,C46/E46)</f>
+        <v>6.76847488524102</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>12.55</v>
+      </c>
+      <c r="H46" s="26" t="s">
+        <v>197</v>
+      </c>
+      <c r="I46" s="16" t="n">
+        <f aca="false">C46*$C$36</f>
+        <v>108.295598163856</v>
+      </c>
+      <c r="J46" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H46,$A$42:$A$58,0))=0,0,I46/INDEX($E$42:$E$58,MATCH($H46,$A$42:$A$58,0)))</f>
+        <v>6.76847488524102</v>
+      </c>
+      <c r="K46" s="16" t="n">
+        <f aca="false">C46*G46+I46*INDEX($G$42:$G$58,MATCH($H46,$A$42:$A$58,0))+(F46+J46)*$C$37</f>
+        <v>3530.43650014171</v>
+      </c>
+      <c r="L46" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D46,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M46" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H46,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="B47" s="16" t="n">
+        <f aca="false">INDEX($B$8:$K$8,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>1604.4414</v>
+      </c>
+      <c r="C47" s="16" t="n">
+        <f aca="false">B47*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>20.5606157082375</v>
+      </c>
+      <c r="D47" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E47" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D47,$A$25:$A$32,0))</f>
+        <v>16</v>
+      </c>
+      <c r="F47" s="17" t="n">
+        <f aca="false">IF(E47=0,0,C47/E47)</f>
+        <v>1.28503848176484</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="H47" s="26" t="s">
+        <v>198</v>
+      </c>
+      <c r="I47" s="16" t="n">
+        <f aca="false">C47*$C$36</f>
+        <v>20.5606157082375</v>
+      </c>
+      <c r="J47" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H47,$A$42:$A$58,0))=0,0,I47/INDEX($E$42:$E$58,MATCH($H47,$A$42:$A$58,0)))</f>
+        <v>1.28503848176484</v>
+      </c>
+      <c r="K47" s="16" t="n">
+        <f aca="false">C47*G47+I47*INDEX($G$42:$G$58,MATCH($H47,$A$42:$A$58,0))+(F47+J47)*$C$37</f>
+        <v>672.332133659366</v>
+      </c>
+      <c r="L47" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D47,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M47" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H47,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B48" s="16" t="n">
+        <f aca="false">INDEX($B$9:$K$9,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>836.3508</v>
+      </c>
+      <c r="C48" s="16" t="n">
+        <f aca="false">B48*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>10.717678686225</v>
+      </c>
+      <c r="D48" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="E48" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D48,$A$25:$A$32,0))</f>
+        <v>2</v>
+      </c>
+      <c r="F48" s="17" t="n">
+        <f aca="false">IF(E48=0,0,C48/E48)</f>
+        <v>5.3588393431125</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H48" s="26" t="s">
+        <v>199</v>
+      </c>
+      <c r="I48" s="16" t="n">
+        <f aca="false">C48*$C$36</f>
+        <v>10.717678686225</v>
+      </c>
+      <c r="J48" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H48,$A$42:$A$58,0))=0,0,I48/INDEX($E$42:$E$58,MATCH($H48,$A$42:$A$58,0)))</f>
+        <v>5.3588393431125</v>
+      </c>
+      <c r="K48" s="16" t="n">
+        <f aca="false">C48*G48+I48*INDEX($G$42:$G$58,MATCH($H48,$A$42:$A$58,0))+(F48+J48)*$C$37</f>
+        <v>2786.5964584185</v>
+      </c>
+      <c r="L48" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D48,$A$25:$A$32,0))</f>
+        <v>R</v>
+      </c>
+      <c r="M48" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H48,$A$42:$A$58,0))</f>
+        <v>R</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="B49" s="16" t="n">
+        <f aca="false">INDEX($B$10:$K$10,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>483.4792</v>
+      </c>
+      <c r="C49" s="16" t="n">
+        <f aca="false">B49*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>6.19569529565</v>
+      </c>
+      <c r="D49" s="25" t="s">
+        <v>222</v>
+      </c>
+      <c r="E49" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D49,$A$25:$A$32,0))</f>
+        <v>24</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <f aca="false">IF(E49=0,0,C49/E49)</f>
+        <v>0.258153970652083</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H49" s="26" t="s">
+        <v>200</v>
+      </c>
+      <c r="I49" s="16" t="n">
+        <f aca="false">C49*$C$36</f>
+        <v>6.19569529565</v>
+      </c>
+      <c r="J49" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H49,$A$42:$A$58,0))=0,0,I49/INDEX($E$42:$E$58,MATCH($H49,$A$42:$A$58,0)))</f>
+        <v>0.258153970652083</v>
+      </c>
+      <c r="K49" s="16" t="n">
+        <f aca="false">C49*G49+I49*INDEX($G$42:$G$58,MATCH($H49,$A$42:$A$58,0))+(F49+J49)*$C$37</f>
+        <v>136.3052965043</v>
+      </c>
+      <c r="L49" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D49,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M49" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H49,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="B50" s="16" t="n">
+        <f aca="false">INDEX($B$11:$K$11,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>4167.5596</v>
+      </c>
+      <c r="C50" s="16" t="n">
+        <f aca="false">B50*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>53.406494856575</v>
+      </c>
+      <c r="D50" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E50" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D50,$A$25:$A$32,0))</f>
+        <v>16</v>
+      </c>
+      <c r="F50" s="17" t="n">
+        <f aca="false">IF(E50=0,0,C50/E50)</f>
+        <v>3.33790592853594</v>
+      </c>
+      <c r="G50" s="7" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="H50" s="26" t="s">
+        <v>201</v>
+      </c>
+      <c r="I50" s="16" t="n">
+        <f aca="false">C50*$C$36</f>
+        <v>53.406494856575</v>
+      </c>
+      <c r="J50" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H50,$A$42:$A$58,0))=0,0,I50/INDEX($E$42:$E$58,MATCH($H50,$A$42:$A$58,0)))</f>
+        <v>3.33790592853594</v>
+      </c>
+      <c r="K50" s="16" t="n">
+        <f aca="false">C50*G50+I50*INDEX($G$42:$G$58,MATCH($H50,$A$42:$A$58,0))+(F50+J50)*$C$37</f>
+        <v>1281.7558765578</v>
+      </c>
+      <c r="L50" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D50,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M50" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H50,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="B51" s="16" t="n">
+        <f aca="false">INDEX($B$12:$K$12,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>22734.5017</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <f aca="false">B51*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>291.338376566431</v>
+      </c>
+      <c r="D51" s="25" t="s">
+        <v>219</v>
+      </c>
+      <c r="E51" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D51,$A$25:$A$32,0))</f>
+        <v>30</v>
+      </c>
+      <c r="F51" s="17" t="n">
+        <f aca="false">IF(E51=0,0,C51/E51)</f>
+        <v>9.71127921888104</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="H51" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="I51" s="16" t="n">
+        <f aca="false">C51*$C$36</f>
+        <v>291.338376566431</v>
+      </c>
+      <c r="J51" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H51,$A$42:$A$58,0))=0,0,I51/INDEX($E$42:$E$58,MATCH($H51,$A$42:$A$58,0)))</f>
+        <v>18.208648535402</v>
+      </c>
+      <c r="K51" s="16" t="n">
+        <f aca="false">C51*G51+I51*INDEX($G$42:$G$58,MATCH($H51,$A$42:$A$58,0))+(F51+J51)*$C$37</f>
+        <v>10124.0085856835</v>
+      </c>
+      <c r="L51" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D51,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M51" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H51,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="B52" s="16" t="n">
+        <f aca="false">INDEX($B$13:$K$13,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>7769.5771</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <f aca="false">B52*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>99.5656737407937</v>
+      </c>
+      <c r="D52" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E52" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D52,$A$25:$A$32,0))</f>
+        <v>16</v>
+      </c>
+      <c r="F52" s="17" t="n">
+        <f aca="false">IF(E52=0,0,C52/E52)</f>
+        <v>6.22285460879961</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="H52" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="I52" s="16" t="n">
+        <f aca="false">C52*$C$36</f>
+        <v>99.5656737407937</v>
+      </c>
+      <c r="J52" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H52,$A$42:$A$58,0))=0,0,I52/INDEX($E$42:$E$58,MATCH($H52,$A$42:$A$58,0)))</f>
+        <v>6.22285460879961</v>
+      </c>
+      <c r="K52" s="16" t="n">
+        <f aca="false">C52*G52+I52*INDEX($G$42:$G$58,MATCH($H52,$A$42:$A$58,0))+(F52+J52)*$C$37</f>
+        <v>4729.3695026877</v>
+      </c>
+      <c r="L52" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D52,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M52" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H52,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="B53" s="16" t="n">
+        <f aca="false">INDEX($B$14:$K$14,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>1271.9411</v>
+      </c>
+      <c r="C53" s="16" t="n">
+        <f aca="false">B53*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>16.2996867075438</v>
+      </c>
+      <c r="D53" s="25" t="s">
+        <v>222</v>
+      </c>
+      <c r="E53" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D53,$A$25:$A$32,0))</f>
+        <v>24</v>
+      </c>
+      <c r="F53" s="17" t="n">
+        <f aca="false">IF(E53=0,0,C53/E53)</f>
+        <v>0.679153612814323</v>
+      </c>
+      <c r="G53" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="H53" s="26" t="s">
+        <v>204</v>
+      </c>
+      <c r="I53" s="16" t="n">
+        <f aca="false">C53*$C$36</f>
+        <v>16.2996867075438</v>
+      </c>
+      <c r="J53" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H53,$A$42:$A$58,0))=0,0,I53/INDEX($E$42:$E$58,MATCH($H53,$A$42:$A$58,0)))</f>
+        <v>0.679153612814323</v>
+      </c>
+      <c r="K53" s="16" t="n">
+        <f aca="false">C53*G53+I53*INDEX($G$42:$G$58,MATCH($H53,$A$42:$A$58,0))+(F53+J53)*$C$37</f>
+        <v>358.593107565962</v>
+      </c>
+      <c r="L53" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D53,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M53" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H53,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B54" s="16" t="n">
+        <f aca="false">INDEX($B$15:$K$15,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>436.6868</v>
+      </c>
+      <c r="C54" s="16" t="n">
+        <f aca="false">B54*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>5.596059463225</v>
+      </c>
+      <c r="D54" s="25" t="s">
+        <v>223</v>
+      </c>
+      <c r="E54" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D54,$A$25:$A$32,0))</f>
+        <v>16</v>
+      </c>
+      <c r="F54" s="17" t="n">
+        <f aca="false">IF(E54=0,0,C54/E54)</f>
+        <v>0.349753716451563</v>
+      </c>
+      <c r="G54" s="7" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H54" s="26" t="s">
+        <v>205</v>
+      </c>
+      <c r="I54" s="16" t="n">
+        <f aca="false">C54*$C$36</f>
+        <v>5.596059463225</v>
+      </c>
+      <c r="J54" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H54,$A$42:$A$58,0))=0,0,I54/INDEX($E$42:$E$58,MATCH($H54,$A$42:$A$58,0)))</f>
+        <v>0.349753716451563</v>
+      </c>
+      <c r="K54" s="16" t="n">
+        <f aca="false">C54*G54+I54*INDEX($G$42:$G$58,MATCH($H54,$A$42:$A$58,0))+(F54+J54)*$C$37</f>
+        <v>226.640408260613</v>
+      </c>
+      <c r="L54" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D54,$A$25:$A$32,0))</f>
+        <v>B</v>
+      </c>
+      <c r="M54" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H54,$A$42:$A$58,0))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="12" t="s">
+        <v>206</v>
+      </c>
+      <c r="B55" s="16" t="n">
+        <f aca="false">INDEX($B$16:$K$16,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>1041.9397</v>
+      </c>
+      <c r="C55" s="16" t="n">
+        <f aca="false">B55*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>13.3522618918062</v>
+      </c>
+      <c r="D55" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="E55" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D55,$A$25:$A$32,0))</f>
+        <v>2</v>
+      </c>
+      <c r="F55" s="17" t="n">
+        <f aca="false">IF(E55=0,0,C55/E55)</f>
+        <v>6.67613094590312</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <v>55</v>
+      </c>
+      <c r="H55" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="I55" s="16" t="n">
+        <f aca="false">C55*$C$36</f>
+        <v>13.3522618918062</v>
+      </c>
+      <c r="J55" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H55,$A$42:$A$58,0))=0,0,I55/INDEX($E$42:$E$58,MATCH($H55,$A$42:$A$58,0)))</f>
+        <v>6.67613094590312</v>
+      </c>
+      <c r="K55" s="16" t="n">
+        <f aca="false">C55*G55+I55*INDEX($G$42:$G$58,MATCH($H55,$A$42:$A$58,0))+(F55+J55)*$C$37</f>
+        <v>2870.73630673834</v>
+      </c>
+      <c r="L55" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D55,$A$25:$A$32,0))</f>
+        <v>R</v>
+      </c>
+      <c r="M55" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H55,$A$42:$A$58,0))</f>
+        <v>R</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B56" s="16" t="n">
+        <f aca="false">INDEX($B$17:$K$17,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>2292.2673</v>
+      </c>
+      <c r="C56" s="16" t="n">
+        <f aca="false">B56*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>29.3749756493812</v>
+      </c>
+      <c r="D56" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="E56" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D56,$A$25:$A$32,0))</f>
+        <v>2</v>
+      </c>
+      <c r="F56" s="17" t="n">
+        <f aca="false">IF(E56=0,0,C56/E56)</f>
+        <v>14.6874878246906</v>
+      </c>
+      <c r="G56" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H56" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="I56" s="16" t="n">
+        <f aca="false">C56*$C$36</f>
+        <v>29.3749756493812</v>
+      </c>
+      <c r="J56" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H56,$A$42:$A$58,0))=0,0,I56/INDEX($E$42:$E$58,MATCH($H56,$A$42:$A$58,0)))</f>
+        <v>14.6874878246906</v>
+      </c>
+      <c r="K56" s="16" t="n">
+        <f aca="false">C56*G56+I56*INDEX($G$42:$G$58,MATCH($H56,$A$42:$A$58,0))+(F56+J56)*$C$37</f>
+        <v>7637.49366883912</v>
+      </c>
+      <c r="L56" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D56,$A$25:$A$32,0))</f>
+        <v>R</v>
+      </c>
+      <c r="M56" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H56,$A$42:$A$58,0))</f>
+        <v>R</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="12" t="s">
+        <v>208</v>
+      </c>
+      <c r="B57" s="16" t="n">
+        <f aca="false">INDEX($B$18:$K$18,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>500.1311</v>
+      </c>
+      <c r="C57" s="16" t="n">
+        <f aca="false">B57*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>6.40908627191875</v>
+      </c>
+      <c r="D57" s="25" t="s">
+        <v>228</v>
+      </c>
+      <c r="E57" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D57,$A$25:$A$32,0))</f>
+        <v>1</v>
+      </c>
+      <c r="F57" s="17" t="n">
+        <f aca="false">IF(E57=0,0,C57/E57)</f>
+        <v>6.40908627191875</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>140</v>
+      </c>
+      <c r="H57" s="26" t="s">
+        <v>209</v>
+      </c>
+      <c r="I57" s="16" t="n">
+        <f aca="false">C57*$C$36</f>
+        <v>6.40908627191875</v>
+      </c>
+      <c r="J57" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H57,$A$42:$A$58,0))=0,0,I57/INDEX($E$42:$E$58,MATCH($H57,$A$42:$A$58,0)))</f>
+        <v>6.40908627191875</v>
+      </c>
+      <c r="K57" s="16" t="n">
+        <f aca="false">C57*G57+I57*INDEX($G$42:$G$58,MATCH($H57,$A$42:$A$58,0))+(F57+J57)*$C$37</f>
+        <v>2852.04339100384</v>
+      </c>
+      <c r="L57" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D57,$A$25:$A$32,0))</f>
+        <v>R</v>
+      </c>
+      <c r="M57" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H57,$A$42:$A$58,0))</f>
+        <v>R</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B58" s="16" t="n">
+        <f aca="false">INDEX($B$19:$K$19,MATCH(Datos!$C$3,$B$2:$K$2,0))</f>
+        <v>333.4207</v>
+      </c>
+      <c r="C58" s="16" t="n">
+        <f aca="false">B58*INDEX($B$20:$K$20,MATCH(Datos!$C$3,$B$2:$K$2,0))/(12*Datos!$C$4)</f>
+        <v>4.27272375411875</v>
+      </c>
+      <c r="D58" s="25" t="s">
+        <v>229</v>
+      </c>
+      <c r="E58" s="16" t="n">
+        <f aca="false">INDEX($C$25:$C$32,MATCH(D58,$A$25:$A$32,0))</f>
+        <v>1</v>
+      </c>
+      <c r="F58" s="17" t="n">
+        <f aca="false">IF(E58=0,0,C58/E58)</f>
+        <v>4.27272375411875</v>
+      </c>
+      <c r="G58" s="7" t="n">
+        <v>185</v>
+      </c>
+      <c r="H58" s="26" t="s">
+        <v>209</v>
+      </c>
+      <c r="I58" s="16" t="n">
+        <f aca="false">C58*$C$36</f>
+        <v>4.27272375411875</v>
+      </c>
+      <c r="J58" s="17" t="n">
+        <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H58,$A$42:$A$58,0))=0,0,I58/INDEX($E$42:$E$58,MATCH($H58,$A$42:$A$58,0)))</f>
+        <v>4.27272375411875</v>
+      </c>
+      <c r="K58" s="16" t="n">
+        <f aca="false">C58*G58+I58*INDEX($G$42:$G$58,MATCH($H58,$A$42:$A$58,0))+(F58+J58)*$C$37</f>
+        <v>2093.63463951819</v>
+      </c>
+      <c r="L58" s="4" t="str">
+        <f aca="false">INDEX($B$25:$B$32,MATCH(D58,$A$25:$A$32,0))</f>
+        <v>R</v>
+      </c>
+      <c r="M58" s="4" t="str">
+        <f aca="false">INDEX($L$42:$L$58,MATCH($H58,$A$42:$A$58,0))</f>
+        <v>R</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B59" s="13" t="n">
+        <f aca="false">SUM(B42:B58)</f>
+        <v>371907.6896</v>
+      </c>
+      <c r="C59" s="13" t="n">
+        <f aca="false">SUM(C42:C58)</f>
+        <v>4765.9273095322</v>
+      </c>
+      <c r="F59" s="13" t="n">
+        <f aca="false">SUM(F42:F58)</f>
+        <v>166.825819872505</v>
+      </c>
+      <c r="I59" s="13" t="n">
+        <f aca="false">SUM(I42:I58)</f>
+        <v>4765.9273095322</v>
+      </c>
+      <c r="J59" s="13" t="n">
+        <f aca="false">SUM(J42:J58)</f>
+        <v>246.968285295459</v>
+      </c>
+      <c r="K59" s="13" t="n">
+        <f aca="false">SUM(K42:K58)</f>
+        <v>109200.466684414</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+      <c r="J60" s="3"/>
+      <c r="K60" s="3"/>
+      <c r="L60" s="3"/>
+      <c r="M60" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A21:M21"/>
+    <mergeCell ref="D24:M24"/>
+    <mergeCell ref="D25:M25"/>
+    <mergeCell ref="D26:M26"/>
+    <mergeCell ref="D27:M27"/>
+    <mergeCell ref="D28:M28"/>
+    <mergeCell ref="D29:M29"/>
+    <mergeCell ref="D30:M30"/>
+    <mergeCell ref="D31:M31"/>
+    <mergeCell ref="D32:M32"/>
+    <mergeCell ref="D35:M35"/>
+    <mergeCell ref="D36:M36"/>
+    <mergeCell ref="D37:M37"/>
+    <mergeCell ref="D38:M38"/>
+    <mergeCell ref="A60:M60"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="16" t="n">
+        <f aca="false">SUMIF(Recargas!$L$42:$L$58,"A",Recargas!$F$42:$F$58)</f>
+        <v>34.9350816432777</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <f aca="false">SUMIF(Recargas!$L$42:$L$58,"B",Recargas!$F$42:$F$58)</f>
+        <v>94.4864700894838</v>
+      </c>
+      <c r="E4" s="16" t="n">
+        <f aca="false">SUMIF(Recargas!$L$42:$L$58,"R",Recargas!$F$42:$F$58)</f>
+        <v>37.4042681397438</v>
+      </c>
+      <c r="F4" s="16" t="n">
+        <f aca="false">SUMPRODUCT(Recargas!$C$42:$C$58,Recargas!$G$42:$G$58)+SUM(Recargas!$F$42:$F$58)*Recargas!$C$37</f>
+        <v>41433.0582964252</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>256</v>
+      </c>
+      <c r="B5" s="4"/>
+      <c r="C5" s="13" t="n">
+        <f aca="false">SUMIF(Recargas!$L$42:$L$58,"A",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"A",Recargas!$J$42:$J$58)</f>
+        <v>34.9350816432777</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <f aca="false">SUMIF(Recargas!$L$42:$L$58,"B",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"B",Recargas!$J$42:$J$58)</f>
+        <v>304.050487245199</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <f aca="false">SUMIF(Recargas!$L$42:$L$58,"R",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"R",Recargas!$J$42:$J$58)</f>
+        <v>74.8085362794875</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <f aca="false">Recargas!K59</f>
+        <v>109200.466684414</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <f aca="false">C4/C3</f>
+        <v>3.88167573814197</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <f aca="false">D4/D3</f>
+        <v>11.8108087611855</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <f aca="false">E4/E3</f>
+        <v>18.7021340698719</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <f aca="false">F4/F3</f>
+        <v>20.7165291482126</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <f aca="false">C5/C3</f>
+        <v>3.88167573814197</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <f aca="false">D5/D3</f>
+        <v>38.0063109056499</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <f aca="false">E5/E3</f>
+        <v>37.4042681397438</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <f aca="false">F5/F3</f>
+        <v>54.600233342207</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <f aca="false">MAX(C6:F6)</f>
+        <v>20.7165291482126</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="18" t="n">
+        <f aca="false">MAX(C7:F7)</f>
+        <v>54.600233342207</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>260</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <f aca="false">C10/Recargas!$C$38</f>
+        <v>10.9200466684414</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="C12" s="13" t="n">
+        <f aca="false">ROUNDUP(C11,0)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4" t="str">
+        <f aca="false">INDEX(C2:F2,MATCH(C10,C7:F7,0))</f>
+        <v>Peso (kg)</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <f aca="false">C3*INDEX(Recargas!$C$25:$C$32,MATCH("A 1 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 1 kg",Recargas!$A$42:$A$58,0))</f>
+        <v>1231.2</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="13" t="n">
+        <f aca="false">C15+D3*INDEX(Recargas!$C$25:$C$32,MATCH("B 5 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 5 kg",Recargas!$A$42:$A$58,0))+E3*INDEX(Recargas!$C$25:$C$32,MATCH("R 50 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 50 kg s/ruedas",Recargas!$A$42:$A$58,0))+(C3+D3+E3)*Recargas!$C$37</f>
+        <v>4403.2</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>266</v>
+      </c>
+      <c r="B17" s="4"/>
+      <c r="C17" s="22" t="str">
+        <f aca="false">IF(C16&lt;=F3,"sí","no")</f>
+        <v>no</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:F19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Palletizado recargas: jaulas B de 2 pisos y comparación de vehículos
Las jaulas tipo B llevan 2 pisos (el Word admite más de uno). La hoja
Recargas_camion compara el Iveco del Word, el camión chico y el sider
por lugares y por peso, y elige el de menos viajes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/palletizado_PT.xlsx
+++ b/salida/palletizado_PT.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="280">
   <si>
     <t xml:space="preserve">General</t>
   </si>
@@ -673,6 +673,12 @@
     <t xml:space="preserve">Clase</t>
   </si>
   <si>
+    <t xml:space="preserve">Por piso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pisos</t>
+  </si>
+  <si>
     <t xml:space="preserve">U por jaula</t>
   </si>
   <si>
@@ -691,15 +697,21 @@
     <t xml:space="preserve">B</t>
   </si>
   <si>
-    <t xml:space="preserve">Tipo B multiformato</t>
+    <t xml:space="preserve">Tipo B multiformato: 30 por piso. 2 pisos (Word: «se puede hacer más de un piso»); 2 cajas de 10 kg de Datos = 1.370 mm ≤ 1.455 mm (criterio)</t>
   </si>
   <si>
     <t xml:space="preserve">B 5 kg</t>
   </si>
   <si>
+    <t xml:space="preserve">Tipo B multiformato: 24 por piso. 2 pisos (Word: «se puede hacer más de un piso»); 2 cajas de 10 kg de Datos = 1.370 mm ≤ 1.455 mm (criterio)</t>
+  </si>
+  <si>
     <t xml:space="preserve">B 10 kg</t>
   </si>
   <si>
+    <t xml:space="preserve">Tipo B multiformato: 16 por piso. 2 pisos (Word: «se puede hacer más de un piso»); 2 cajas de 10 kg de Datos = 1.370 mm ≤ 1.455 mm (criterio)</t>
+  </si>
+  <si>
     <t xml:space="preserve">R 25 kg</t>
   </si>
   <si>
@@ -775,49 +787,73 @@
     <t xml:space="preserve">Fuentes: formato, Word (ABC) y por tamaño el resto (criterio); peso, FLAMA_BOM hoja Resumen (peso de catálogo); sustituto, Reservas y Sustitutos filas 54 a 65.</t>
   </si>
   <si>
-    <t xml:space="preserve">Camión de recargas: Iveco cabina simple con baranda rebatible (Word Proceso de recargas, Recepción y registro)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jaulas tipo A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jaulas tipo B</t>
+    <t xml:space="preserve">Recargas y sustitutos de la planta industrial: lugares, peso y viajes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por semana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jaulas B</t>
   </si>
   <si>
     <t xml:space="preserve">Pallets rodantes</t>
   </si>
   <si>
+    <t xml:space="preserve">Lugares</t>
+  </si>
+  <si>
     <t xml:space="preserve">Peso (kg)</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacidad por viaje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo recargados por semana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recargados + sustitutos por semana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viajes por semana: solo recargados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viajes por semana: con sustitutos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VIAJES POR SEMANA (con sustitutos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Viajes por día hábil (con sustitutos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Camiones para 1 viaje por día</t>
+    <t xml:space="preserve">Solo recargados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargados + sustitutos (máximo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehículo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lugares por viaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carga útil (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viajes/sem por lugar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viajes/sem por peso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viajes por día</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Iveco cabina simple del Word (9 A + 8 B + 2 rodantes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camión chico: GyL baranda volcable 4,30 m (Accelo 1016)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sider GyL Full para balancín 7,50 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehículo con menos viajes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camiones con ese vehículo (1 viaje por día cada uno)</t>
   </si>
   <si>
     <t xml:space="preserve">camiones</t>
   </si>
   <si>
-    <t xml:space="preserve">Limita</t>
+    <t xml:space="preserve">Control del pico de 1,2 t del Word</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viaje del Word</t>
   </si>
   <si>
     <t xml:space="preserve">Peso de 9 jaulas A llenas de 1 kg</t>
@@ -829,7 +865,7 @@
     <t xml:space="preserve">¿Entra en la carga útil?</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuente de la capacidad: 9 jaulas tipo A, 8 tipo B, 2 pallets de rodantes y unas 2 t de carga útil, con un pico de 1,2 t (Word Proceso de recargas, Recepción y registro).</t>
+    <t xml:space="preserve">Fuentes: Iveco, 9 jaulas A, 8 jaulas B, 2 pallets de rodantes, unas 2 t y pico de 1,2 t (Word Proceso de recargas, Recepción y registro). Camión chico y sider: hojas Datos y Camion.</t>
   </si>
 </sst>
 </file>
@@ -974,7 +1010,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1080,6 +1116,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9285,10 +9325,14 @@
         <v>215</v>
       </c>
       <c r="D24" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="F24" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -9299,19 +9343,24 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
+      <c r="D25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <f aca="false">C25*D25</f>
+        <v>72</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>220</v>
+      </c>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
@@ -9320,21 +9369,26 @@
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
+      <c r="D26" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <f aca="false">C26*D26</f>
+        <v>60</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>223</v>
+      </c>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
@@ -9343,21 +9397,26 @@
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>222</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="C27" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
+      <c r="D27" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <f aca="false">C27*D27</f>
+        <v>48</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>225</v>
+      </c>
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
@@ -9366,21 +9425,26 @@
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
+      <c r="D28" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <f aca="false">C28*D28</f>
+        <v>32</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>227</v>
+      </c>
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -9391,20 +9455,25 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C29" s="16" t="n">
         <f aca="false">MAX(INT(Datos!$C$8/Datos!$C$34)*INT(Datos!$C$9/Datos!$C$35),INT(Datos!$C$8/Datos!$C$35)*INT(Datos!$C$9/Datos!$C$34))</f>
         <v>2</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
+      <c r="D29" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <f aca="false">C29*D29</f>
+        <v>2</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>230</v>
+      </c>
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
@@ -9415,20 +9484,25 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C30" s="16" t="n">
         <f aca="false">MAX(INT(Datos!$C$8/Datos!$D$34)*INT(Datos!$C$9/Datos!$D$35),INT(Datos!$C$8/Datos!$D$35)*INT(Datos!$C$9/Datos!$D$34))</f>
         <v>2</v>
       </c>
-      <c r="D30" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
+      <c r="D30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <f aca="false">C30*D30</f>
+        <v>2</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>230</v>
+      </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
@@ -9439,20 +9513,25 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C31" s="16" t="n">
         <f aca="false">MAX(INT(Datos!$C$8/Datos!$E$34)*INT(Datos!$C$9/Datos!$E$35),INT(Datos!$C$8/Datos!$E$35)*INT(Datos!$C$9/Datos!$E$34))</f>
         <v>1</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
+      <c r="D31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <f aca="false">C31*D31</f>
+        <v>1</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>230</v>
+      </c>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
@@ -9463,20 +9542,25 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>229</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>225</v>
       </c>
       <c r="C32" s="16" t="n">
         <f aca="false">MAX(INT(Datos!$C$8/Datos!$F$34)*INT(Datos!$C$9/Datos!$F$35),INT(Datos!$C$8/Datos!$F$35)*INT(Datos!$C$9/Datos!$F$34))</f>
         <v>1</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
+      <c r="D32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <f aca="false">C32*D32</f>
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>230</v>
+      </c>
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
@@ -9487,7 +9571,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9515,7 +9599,7 @@
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>165</v>
@@ -9524,7 +9608,7 @@
         <v>1</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -9538,7 +9622,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>18</v>
@@ -9547,7 +9631,7 @@
         <v>60</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -9561,16 +9645,16 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>5</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -9584,7 +9668,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9592,40 +9676,40 @@
         <v>192</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D41" s="2" t="s">
         <v>213</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>214</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9641,10 +9725,10 @@
         <v>2515.32587831599</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E42" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D42,$A$25:$A$32,0))</f>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D42,$A$25:$A$32,0))</f>
         <v>72</v>
       </c>
       <c r="F42" s="17" t="n">
@@ -9663,11 +9747,11 @@
       </c>
       <c r="J42" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H42,$A$42:$A$58,0))=0,0,I42/INDEX($E$42:$E$58,MATCH($H42,$A$42:$A$58,0)))</f>
-        <v>104.805244929833</v>
+        <v>52.4026224649165</v>
       </c>
       <c r="K42" s="16" t="n">
         <f aca="false">C42*G42+I42*INDEX($G$42:$G$58,MATCH($H42,$A$42:$A$58,0))+(F42+J42)*$C$37</f>
-        <v>34543.808728873</v>
+        <v>31399.651380978</v>
       </c>
       <c r="L42" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D42,$A$25:$A$32,0))</f>
@@ -9691,15 +9775,15 @@
         <v>212.991938385275</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E43" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D43,$A$25:$A$32,0))</f>
-        <v>30</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D43,$A$25:$A$32,0))</f>
+        <v>60</v>
       </c>
       <c r="F43" s="17" t="n">
         <f aca="false">IF(E43=0,0,C43/E43)</f>
-        <v>7.09973127950917</v>
+        <v>3.54986563975458</v>
       </c>
       <c r="G43" s="7" t="n">
         <v>4.6</v>
@@ -9713,11 +9797,11 @@
       </c>
       <c r="J43" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H43,$A$42:$A$58,0))=0,0,I43/INDEX($E$42:$E$58,MATCH($H43,$A$42:$A$58,0)))</f>
-        <v>8.87466409938646</v>
+        <v>4.43733204969323</v>
       </c>
       <c r="K43" s="16" t="n">
         <f aca="false">C43*G43+I43*INDEX($G$42:$G$58,MATCH($H43,$A$42:$A$58,0))+(F43+J43)*$C$37</f>
-        <v>3748.65811558084</v>
+        <v>3269.42625421397</v>
       </c>
       <c r="L43" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D43,$A$25:$A$32,0))</f>
@@ -9741,15 +9825,15 @@
         <v>1295.51572765746</v>
       </c>
       <c r="D44" s="25" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E44" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D44,$A$25:$A$32,0))</f>
-        <v>24</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D44,$A$25:$A$32,0))</f>
+        <v>48</v>
       </c>
       <c r="F44" s="17" t="n">
         <f aca="false">IF(E44=0,0,C44/E44)</f>
-        <v>53.9798219857276</v>
+        <v>26.9899109928638</v>
       </c>
       <c r="G44" s="7" t="n">
         <v>8.5</v>
@@ -9763,11 +9847,11 @@
       </c>
       <c r="J44" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H44,$A$42:$A$58,0))=0,0,I44/INDEX($E$42:$E$58,MATCH($H44,$A$42:$A$58,0)))</f>
-        <v>53.9798219857276</v>
+        <v>26.9899109928638</v>
       </c>
       <c r="K44" s="16" t="n">
         <f aca="false">C44*G44+I44*INDEX($G$42:$G$58,MATCH($H44,$A$42:$A$58,0))+(F44+J44)*$C$37</f>
-        <v>28501.3460084642</v>
+        <v>25262.5566893205</v>
       </c>
       <c r="L44" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D44,$A$25:$A$32,0))</f>
@@ -9791,15 +9875,15 @@
         <v>76.7088384177063</v>
       </c>
       <c r="D45" s="25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E45" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D45,$A$25:$A$32,0))</f>
-        <v>16</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D45,$A$25:$A$32,0))</f>
+        <v>32</v>
       </c>
       <c r="F45" s="17" t="n">
         <f aca="false">IF(E45=0,0,C45/E45)</f>
-        <v>4.79430240110664</v>
+        <v>2.39715120055332</v>
       </c>
       <c r="G45" s="7" t="n">
         <v>16.5</v>
@@ -9813,11 +9897,11 @@
       </c>
       <c r="J45" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H45,$A$42:$A$58,0))=0,0,I45/INDEX($E$42:$E$58,MATCH($H45,$A$42:$A$58,0)))</f>
-        <v>4.79430240110664</v>
+        <v>2.39715120055332</v>
       </c>
       <c r="K45" s="16" t="n">
         <f aca="false">C45*G45+I45*INDEX($G$42:$G$58,MATCH($H45,$A$42:$A$58,0))+(F45+J45)*$C$37</f>
-        <v>3106.7079559171</v>
+        <v>2819.04981185071</v>
       </c>
       <c r="L45" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D45,$A$25:$A$32,0))</f>
@@ -9841,15 +9925,15 @@
         <v>108.295598163856</v>
       </c>
       <c r="D46" s="25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E46" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D46,$A$25:$A$32,0))</f>
-        <v>16</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D46,$A$25:$A$32,0))</f>
+        <v>32</v>
       </c>
       <c r="F46" s="17" t="n">
         <f aca="false">IF(E46=0,0,C46/E46)</f>
-        <v>6.76847488524102</v>
+        <v>3.38423744262051</v>
       </c>
       <c r="G46" s="7" t="n">
         <v>12.55</v>
@@ -9863,11 +9947,11 @@
       </c>
       <c r="J46" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H46,$A$42:$A$58,0))=0,0,I46/INDEX($E$42:$E$58,MATCH($H46,$A$42:$A$58,0)))</f>
-        <v>6.76847488524102</v>
+        <v>3.38423744262051</v>
       </c>
       <c r="K46" s="16" t="n">
         <f aca="false">C46*G46+I46*INDEX($G$42:$G$58,MATCH($H46,$A$42:$A$58,0))+(F46+J46)*$C$37</f>
-        <v>3530.43650014171</v>
+        <v>3124.32800702725</v>
       </c>
       <c r="L46" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D46,$A$25:$A$32,0))</f>
@@ -9891,15 +9975,15 @@
         <v>20.5606157082375</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E47" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D47,$A$25:$A$32,0))</f>
-        <v>16</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D47,$A$25:$A$32,0))</f>
+        <v>32</v>
       </c>
       <c r="F47" s="17" t="n">
         <f aca="false">IF(E47=0,0,C47/E47)</f>
-        <v>1.28503848176484</v>
+        <v>0.642519240882422</v>
       </c>
       <c r="G47" s="7" t="n">
         <v>12.6</v>
@@ -9913,11 +9997,11 @@
       </c>
       <c r="J47" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H47,$A$42:$A$58,0))=0,0,I47/INDEX($E$42:$E$58,MATCH($H47,$A$42:$A$58,0)))</f>
-        <v>1.28503848176484</v>
+        <v>0.642519240882422</v>
       </c>
       <c r="K47" s="16" t="n">
         <f aca="false">C47*G47+I47*INDEX($G$42:$G$58,MATCH($H47,$A$42:$A$58,0))+(F47+J47)*$C$37</f>
-        <v>672.332133659366</v>
+        <v>595.229824753475</v>
       </c>
       <c r="L47" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D47,$A$25:$A$32,0))</f>
@@ -9941,10 +10025,10 @@
         <v>10.717678686225</v>
       </c>
       <c r="D48" s="25" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E48" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D48,$A$25:$A$32,0))</f>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D48,$A$25:$A$32,0))</f>
         <v>2</v>
       </c>
       <c r="F48" s="17" t="n">
@@ -9991,15 +10075,15 @@
         <v>6.19569529565</v>
       </c>
       <c r="D49" s="25" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E49" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D49,$A$25:$A$32,0))</f>
-        <v>24</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D49,$A$25:$A$32,0))</f>
+        <v>48</v>
       </c>
       <c r="F49" s="17" t="n">
         <f aca="false">IF(E49=0,0,C49/E49)</f>
-        <v>0.258153970652083</v>
+        <v>0.129076985326042</v>
       </c>
       <c r="G49" s="7" t="n">
         <v>8.5</v>
@@ -10013,11 +10097,11 @@
       </c>
       <c r="J49" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H49,$A$42:$A$58,0))=0,0,I49/INDEX($E$42:$E$58,MATCH($H49,$A$42:$A$58,0)))</f>
-        <v>0.258153970652083</v>
+        <v>0.129076985326042</v>
       </c>
       <c r="K49" s="16" t="n">
         <f aca="false">C49*G49+I49*INDEX($G$42:$G$58,MATCH($H49,$A$42:$A$58,0))+(F49+J49)*$C$37</f>
-        <v>136.3052965043</v>
+        <v>120.816058265175</v>
       </c>
       <c r="L49" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D49,$A$25:$A$32,0))</f>
@@ -10041,15 +10125,15 @@
         <v>53.406494856575</v>
       </c>
       <c r="D50" s="25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E50" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D50,$A$25:$A$32,0))</f>
-        <v>16</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D50,$A$25:$A$32,0))</f>
+        <v>32</v>
       </c>
       <c r="F50" s="17" t="n">
         <f aca="false">IF(E50=0,0,C50/E50)</f>
-        <v>3.33790592853594</v>
+        <v>1.66895296426797</v>
       </c>
       <c r="G50" s="7" t="n">
         <v>8.25</v>
@@ -10063,11 +10147,11 @@
       </c>
       <c r="J50" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H50,$A$42:$A$58,0))=0,0,I50/INDEX($E$42:$E$58,MATCH($H50,$A$42:$A$58,0)))</f>
-        <v>3.33790592853594</v>
+        <v>1.66895296426797</v>
       </c>
       <c r="K50" s="16" t="n">
         <f aca="false">C50*G50+I50*INDEX($G$42:$G$58,MATCH($H50,$A$42:$A$58,0))+(F50+J50)*$C$37</f>
-        <v>1281.7558765578</v>
+        <v>1081.48152084564</v>
       </c>
       <c r="L50" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D50,$A$25:$A$32,0))</f>
@@ -10091,15 +10175,15 @@
         <v>291.338376566431</v>
       </c>
       <c r="D51" s="25" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E51" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D51,$A$25:$A$32,0))</f>
-        <v>30</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D51,$A$25:$A$32,0))</f>
+        <v>60</v>
       </c>
       <c r="F51" s="17" t="n">
         <f aca="false">IF(E51=0,0,C51/E51)</f>
-        <v>9.71127921888104</v>
+        <v>4.85563960944052</v>
       </c>
       <c r="G51" s="7" t="n">
         <v>9</v>
@@ -10113,11 +10197,11 @@
       </c>
       <c r="J51" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H51,$A$42:$A$58,0))=0,0,I51/INDEX($E$42:$E$58,MATCH($H51,$A$42:$A$58,0)))</f>
-        <v>18.208648535402</v>
+        <v>9.10432426770098</v>
       </c>
       <c r="K51" s="16" t="n">
         <f aca="false">C51*G51+I51*INDEX($G$42:$G$58,MATCH($H51,$A$42:$A$58,0))+(F51+J51)*$C$37</f>
-        <v>10124.0085856835</v>
+        <v>9286.410753055</v>
       </c>
       <c r="L51" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D51,$A$25:$A$32,0))</f>
@@ -10141,15 +10225,15 @@
         <v>99.5656737407937</v>
       </c>
       <c r="D52" s="25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E52" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D52,$A$25:$A$32,0))</f>
-        <v>16</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D52,$A$25:$A$32,0))</f>
+        <v>32</v>
       </c>
       <c r="F52" s="17" t="n">
         <f aca="false">IF(E52=0,0,C52/E52)</f>
-        <v>6.22285460879961</v>
+        <v>3.1114273043998</v>
       </c>
       <c r="G52" s="7" t="n">
         <v>20</v>
@@ -10163,11 +10247,11 @@
       </c>
       <c r="J52" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H52,$A$42:$A$58,0))=0,0,I52/INDEX($E$42:$E$58,MATCH($H52,$A$42:$A$58,0)))</f>
-        <v>6.22285460879961</v>
+        <v>3.1114273043998</v>
       </c>
       <c r="K52" s="16" t="n">
         <f aca="false">C52*G52+I52*INDEX($G$42:$G$58,MATCH($H52,$A$42:$A$58,0))+(F52+J52)*$C$37</f>
-        <v>4729.3695026877</v>
+        <v>4355.99822615973</v>
       </c>
       <c r="L52" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D52,$A$25:$A$32,0))</f>
@@ -10191,15 +10275,15 @@
         <v>16.2996867075438</v>
       </c>
       <c r="D53" s="25" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="E53" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D53,$A$25:$A$32,0))</f>
-        <v>24</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D53,$A$25:$A$32,0))</f>
+        <v>48</v>
       </c>
       <c r="F53" s="17" t="n">
         <f aca="false">IF(E53=0,0,C53/E53)</f>
-        <v>0.679153612814323</v>
+        <v>0.339576806407161</v>
       </c>
       <c r="G53" s="7" t="n">
         <v>8.5</v>
@@ -10213,11 +10297,11 @@
       </c>
       <c r="J53" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H53,$A$42:$A$58,0))=0,0,I53/INDEX($E$42:$E$58,MATCH($H53,$A$42:$A$58,0)))</f>
-        <v>0.679153612814323</v>
+        <v>0.339576806407161</v>
       </c>
       <c r="K53" s="16" t="n">
         <f aca="false">C53*G53+I53*INDEX($G$42:$G$58,MATCH($H53,$A$42:$A$58,0))+(F53+J53)*$C$37</f>
-        <v>358.593107565962</v>
+        <v>317.843890797103</v>
       </c>
       <c r="L53" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D53,$A$25:$A$32,0))</f>
@@ -10241,15 +10325,15 @@
         <v>5.596059463225</v>
       </c>
       <c r="D54" s="25" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E54" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D54,$A$25:$A$32,0))</f>
-        <v>16</v>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D54,$A$25:$A$32,0))</f>
+        <v>32</v>
       </c>
       <c r="F54" s="17" t="n">
         <f aca="false">IF(E54=0,0,C54/E54)</f>
-        <v>0.349753716451563</v>
+        <v>0.174876858225781</v>
       </c>
       <c r="G54" s="7" t="n">
         <v>16.5</v>
@@ -10263,11 +10347,11 @@
       </c>
       <c r="J54" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H54,$A$42:$A$58,0))=0,0,I54/INDEX($E$42:$E$58,MATCH($H54,$A$42:$A$58,0)))</f>
-        <v>0.349753716451563</v>
+        <v>0.174876858225781</v>
       </c>
       <c r="K54" s="16" t="n">
         <f aca="false">C54*G54+I54*INDEX($G$42:$G$58,MATCH($H54,$A$42:$A$58,0))+(F54+J54)*$C$37</f>
-        <v>226.640408260613</v>
+        <v>205.655185273519</v>
       </c>
       <c r="L54" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D54,$A$25:$A$32,0))</f>
@@ -10291,10 +10375,10 @@
         <v>13.3522618918062</v>
       </c>
       <c r="D55" s="25" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E55" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D55,$A$25:$A$32,0))</f>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D55,$A$25:$A$32,0))</f>
         <v>2</v>
       </c>
       <c r="F55" s="17" t="n">
@@ -10341,10 +10425,10 @@
         <v>29.3749756493812</v>
       </c>
       <c r="D56" s="25" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E56" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D56,$A$25:$A$32,0))</f>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D56,$A$25:$A$32,0))</f>
         <v>2</v>
       </c>
       <c r="F56" s="17" t="n">
@@ -10391,10 +10475,10 @@
         <v>6.40908627191875</v>
       </c>
       <c r="D57" s="25" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E57" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D57,$A$25:$A$32,0))</f>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D57,$A$25:$A$32,0))</f>
         <v>1</v>
       </c>
       <c r="F57" s="17" t="n">
@@ -10441,10 +10525,10 @@
         <v>4.27272375411875</v>
       </c>
       <c r="D58" s="25" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E58" s="16" t="n">
-        <f aca="false">INDEX($C$25:$C$32,MATCH(D58,$A$25:$A$32,0))</f>
+        <f aca="false">INDEX($E$25:$E$32,MATCH(D58,$A$25:$A$32,0))</f>
         <v>1</v>
       </c>
       <c r="F58" s="17" t="n">
@@ -10492,7 +10576,7 @@
       </c>
       <c r="F59" s="13" t="n">
         <f aca="false">SUM(F42:F58)</f>
-        <v>166.825819872505</v>
+        <v>119.582584827763</v>
       </c>
       <c r="I59" s="13" t="n">
         <f aca="false">SUM(I42:I58)</f>
@@ -10500,16 +10584,16 @@
       </c>
       <c r="J59" s="13" t="n">
         <f aca="false">SUM(J42:J58)</f>
-        <v>246.968285295459</v>
+        <v>142.186276717601</v>
       </c>
       <c r="K59" s="13" t="n">
         <f aca="false">SUM(K42:K58)</f>
-        <v>109200.466684414</v>
+        <v>100078.952067058</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -10527,15 +10611,15 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A21:M21"/>
-    <mergeCell ref="D24:M24"/>
-    <mergeCell ref="D25:M25"/>
-    <mergeCell ref="D26:M26"/>
-    <mergeCell ref="D27:M27"/>
-    <mergeCell ref="D28:M28"/>
-    <mergeCell ref="D29:M29"/>
-    <mergeCell ref="D30:M30"/>
-    <mergeCell ref="D31:M31"/>
-    <mergeCell ref="D32:M32"/>
+    <mergeCell ref="F24:M24"/>
+    <mergeCell ref="F25:M25"/>
+    <mergeCell ref="F26:M26"/>
+    <mergeCell ref="F27:M27"/>
+    <mergeCell ref="F28:M28"/>
+    <mergeCell ref="F29:M29"/>
+    <mergeCell ref="F30:M30"/>
+    <mergeCell ref="F31:M31"/>
+    <mergeCell ref="F32:M32"/>
     <mergeCell ref="D35:M35"/>
     <mergeCell ref="D36:M36"/>
     <mergeCell ref="D37:M37"/>
@@ -10557,252 +10641,325 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="3" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
+      <c r="A2" s="2" t="s">
+        <v>254</v>
+      </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>253</v>
+        <v>258</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="16" t="n">
+      <c r="C3" s="16" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"A",Recargas!$F$42:$F$58)</f>
         <v>34.9350816432777</v>
       </c>
-      <c r="D4" s="16" t="n">
+      <c r="D3" s="16" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"B",Recargas!$F$42:$F$58)</f>
-        <v>94.4864700894838</v>
-      </c>
-      <c r="E4" s="16" t="n">
+        <v>47.2432350447419</v>
+      </c>
+      <c r="E3" s="16" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"R",Recargas!$F$42:$F$58)</f>
         <v>37.4042681397438</v>
       </c>
-      <c r="F4" s="16" t="n">
+      <c r="F3" s="16" t="n">
+        <f aca="false">SUM(C3:E3)</f>
+        <v>119.582584827763</v>
+      </c>
+      <c r="G3" s="16" t="n">
         <f aca="false">SUMPRODUCT(Recargas!$C$42:$C$58,Recargas!$G$42:$G$58)+SUM(Recargas!$F$42:$F$58)*Recargas!$C$37</f>
-        <v>41433.0582964252</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>256</v>
-      </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="13" t="n">
+        <v>38598.4641937406</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="B4" s="4"/>
+      <c r="C4" s="13" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"A",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"A",Recargas!$J$42:$J$58)</f>
         <v>34.9350816432777</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D4" s="13" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"B",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"B",Recargas!$J$42:$J$58)</f>
-        <v>304.050487245199</v>
-      </c>
-      <c r="E5" s="13" t="n">
+        <v>152.025243622599</v>
+      </c>
+      <c r="E4" s="13" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"R",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"R",Recargas!$J$42:$J$58)</f>
         <v>74.8085362794875</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F4" s="13" t="n">
+        <f aca="false">SUM(C4:E4)</f>
+        <v>261.768861545365</v>
+      </c>
+      <c r="G4" s="13" t="n">
         <f aca="false">Recargas!K59</f>
-        <v>109200.466684414</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C6" s="17" t="n">
-        <f aca="false">C4/C3</f>
-        <v>3.88167573814197</v>
-      </c>
-      <c r="D6" s="17" t="n">
-        <f aca="false">D4/D3</f>
-        <v>11.8108087611855</v>
-      </c>
-      <c r="E6" s="17" t="n">
-        <f aca="false">E4/E3</f>
-        <v>18.7021340698719</v>
-      </c>
-      <c r="F6" s="17" t="n">
-        <f aca="false">F4/F3</f>
-        <v>20.7165291482126</v>
+        <v>100078.952067058</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>267</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>258</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C7" s="17" t="n">
-        <f aca="false">C5/C3</f>
-        <v>3.88167573814197</v>
+        <v>268</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>2000</v>
       </c>
       <c r="D7" s="17" t="n">
-        <f aca="false">D5/D3</f>
-        <v>38.0063109056499</v>
+        <f aca="false">IF(B7=0,0,$F$4/B7)</f>
+        <v>13.7773085023876</v>
       </c>
       <c r="E7" s="17" t="n">
-        <f aca="false">E5/E3</f>
-        <v>37.4042681397438</v>
-      </c>
-      <c r="F7" s="17" t="n">
-        <f aca="false">F5/F3</f>
-        <v>54.600233342207</v>
+        <f aca="false">IF(C7=0,0,$G$4/C7)</f>
+        <v>50.039476033529</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <f aca="false">MAX(D7,E7)</f>
+        <v>50.039476033529</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <f aca="false">F7/Recargas!$C$38</f>
+        <v>10.0078952067058</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B8" s="16" t="n">
+        <f aca="false">Camion!C20</f>
+        <v>6</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <f aca="false">Datos!$C$48</f>
+        <v>6000</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <f aca="false">IF(B8=0,0,$F$4/B8)</f>
+        <v>43.6281435908941</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <f aca="false">IF(C8=0,0,$G$4/C8)</f>
+        <v>16.6798253445097</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <f aca="false">MAX(D8,E8)</f>
+        <v>43.6281435908941</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <f aca="false">F8/Recargas!$C$38</f>
+        <v>8.72562871817882</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C9" s="17" t="n">
-        <f aca="false">MAX(C6:F6)</f>
-        <v>20.7165291482126</v>
+        <v>270</v>
+      </c>
+      <c r="B9" s="16" t="n">
+        <f aca="false">Camion!C5</f>
+        <v>14</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <f aca="false">Datos!$C$42</f>
+        <v>12000</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <f aca="false">IF(B9=0,0,$F$4/B9)</f>
+        <v>18.6977758246689</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <f aca="false">IF(C9=0,0,$G$4/C9)</f>
+        <v>8.33991267225484</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <f aca="false">MAX(D9,E9)</f>
+        <v>18.6977758246689</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <f aca="false">F9/Recargas!$C$38</f>
+        <v>3.73955516493378</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C10" s="18" t="n">
-        <f aca="false">MAX(C7:F7)</f>
-        <v>54.600233342207</v>
+        <v>271</v>
+      </c>
+      <c r="B10" s="22" t="str">
+        <f aca="false">INDEX(A7:A9,MATCH(MIN(F7:F9),F7:F9,0))</f>
+        <v>Sider GyL Full para balancín 7,50 m</v>
+      </c>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="18" t="n">
+        <f aca="false">MIN(F7:F9)</f>
+        <v>18.6977758246689</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <f aca="false">MIN(G7:G9)</f>
+        <v>3.73955516493378</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="C11" s="18" t="n">
-        <f aca="false">C10/Recargas!$C$38</f>
-        <v>10.9200466684414</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>261</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>262</v>
-      </c>
-      <c r="C12" s="13" t="n">
-        <f aca="false">ROUNDUP(C11,0)</f>
-        <v>11</v>
+        <v>273</v>
+      </c>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="13" t="n">
+        <f aca="false">ROUNDUP(G10,0)</f>
+        <v>4</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4" t="str">
-        <f aca="false">INDEX(C2:F2,MATCH(C10,C7:F7,0))</f>
-        <v>Peso (kg)</v>
+      <c r="A13" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="16" t="n">
-        <f aca="false">C3*INDEX(Recargas!$C$25:$C$32,MATCH("A 1 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 1 kg",Recargas!$A$42:$A$58,0))</f>
+        <f aca="false">C14*INDEX(Recargas!$C$25:$C$32,MATCH("A 1 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 1 kg",Recargas!$A$42:$A$58,0))</f>
         <v>1231.2</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>18</v>
       </c>
       <c r="C16" s="13" t="n">
-        <f aca="false">C15+D3*INDEX(Recargas!$C$25:$C$32,MATCH("B 5 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 5 kg",Recargas!$A$42:$A$58,0))+E3*INDEX(Recargas!$C$25:$C$32,MATCH("R 50 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 50 kg s/ruedas",Recargas!$A$42:$A$58,0))+(C3+D3+E3)*Recargas!$C$37</f>
+        <f aca="false">C15+D14*INDEX(Recargas!$C$25:$C$32,MATCH("B 5 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 5 kg",Recargas!$A$42:$A$58,0))+E14*INDEX(Recargas!$C$25:$C$32,MATCH("R 50 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 50 kg s/ruedas",Recargas!$A$42:$A$58,0))+(C14+D14+E14)*Recargas!$C$37</f>
         <v>4403.2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="22" t="str">
-        <f aca="false">IF(C16&lt;=F3,"sí","no")</f>
+        <f aca="false">IF(C16&lt;=F14,"sí","no")</f>
         <v>no</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A19:F19"/>
+  <mergeCells count="2">
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="A19:G19"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Palletizado recargas: máximo de 3 viajes por día y comparación con la demanda
Sustituto de 1 kg para el 1 kg (IRAM 3517-2 9.4.5) y jaula tipo A de 2
pisos: recargados + sustitutos en el sider GyL balancín dan 3 viajes por
día. Tabla que compara por día la demanda de PT, los recargados y los
sustitutos con sus viajes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/palletizado_PT.xlsx
+++ b/salida/palletizado_PT.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="285">
   <si>
     <t xml:space="preserve">General</t>
   </si>
@@ -688,7 +688,7 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">Tipo A: 1 nivel, 8 × 9 celdas de 100 × 140 mm</t>
+    <t xml:space="preserve">Tipo A: 8 × 9 celdas de 100 × 140 mm por piso (el Word la da de 1 nivel). 2 pisos (Word: «se puede hacer más de un piso»); 2 cajas de 1 kg de Datos = 820 mm (criterio)</t>
   </si>
   <si>
     <t xml:space="preserve">B 2,5 kg</t>
@@ -784,7 +784,7 @@
     <t xml:space="preserve">Clase sust.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuentes: formato, Word (ABC) y por tamaño el resto (criterio); peso, FLAMA_BOM hoja Resumen (peso de catálogo); sustituto, Reservas y Sustitutos filas 54 a 65.</t>
+    <t xml:space="preserve">Fuentes: formato, Word (ABC) y por tamaño el resto (criterio); peso, FLAMA_BOM hoja Resumen (peso de catálogo); sustituto, Reservas y Sustitutos filas 54 a 65, salvo el 1 kg: sustituto de 1 kg (IRAM 3517-2 9.4.5: igual clasificación y por lo menos igual capacidad).</t>
   </si>
   <si>
     <t xml:space="preserve">Recargas y sustitutos de la planta industrial: lugares, peso y viajes</t>
@@ -841,13 +841,28 @@
     <t xml:space="preserve">Sider GyL Full para balancín 7,50 m</t>
   </si>
   <si>
-    <t xml:space="preserve">Vehículo con menos viajes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Camiones con ese vehículo (1 viaje por día cada uno)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">camiones</t>
+    <t xml:space="preserve">Máximo de viajes por día</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vehículo elegido (el de menos viajes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿Cumple el máximo de viajes por día?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparación con la demanda (por día hábil)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demanda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matafuegos manuales nuevos (PT, mes pico)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camión chico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recargados de la planta industrial</t>
   </si>
   <si>
     <t xml:space="preserve">Control del pico de 1,2 t del Word</t>
@@ -865,7 +880,7 @@
     <t xml:space="preserve">¿Entra en la carga útil?</t>
   </si>
   <si>
-    <t xml:space="preserve">Fuentes: Iveco, 9 jaulas A, 8 jaulas B, 2 pallets de rodantes, unas 2 t y pico de 1,2 t (Word Proceso de recargas, Recepción y registro). Camión chico y sider: hojas Datos y Camion.</t>
+    <t xml:space="preserve">Fuentes: Iveco, 9 jaulas A, 8 jaulas B, 2 pallets de rodantes, unas 2 t y pico de 1,2 t (Word Proceso de recargas, Recepción y registro). Camión chico y sider: hojas Datos y Camion. Máximo de 3 viajes por día: dato del usuario.</t>
   </si>
 </sst>
 </file>
@@ -1010,7 +1025,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1119,7 +1134,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -9341,7 +9364,7 @@
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
         <v>218</v>
       </c>
@@ -9352,11 +9375,11 @@
         <v>72</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="13" t="n">
         <f aca="false">C25*D25</f>
-        <v>72</v>
+        <v>144</v>
       </c>
       <c r="F25" s="3" t="s">
         <v>220</v>
@@ -9729,17 +9752,17 @@
       </c>
       <c r="E42" s="16" t="n">
         <f aca="false">INDEX($E$25:$E$32,MATCH(D42,$A$25:$A$32,0))</f>
-        <v>72</v>
+        <v>144</v>
       </c>
       <c r="F42" s="17" t="n">
         <f aca="false">IF(E42=0,0,C42/E42)</f>
-        <v>34.9350816432777</v>
+        <v>17.4675408216388</v>
       </c>
       <c r="G42" s="7" t="n">
         <v>1.9</v>
       </c>
       <c r="H42" s="26" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="I42" s="16" t="n">
         <f aca="false">C42*$C$36</f>
@@ -9747,11 +9770,11 @@
       </c>
       <c r="J42" s="17" t="n">
         <f aca="false">IF(INDEX($E$42:$E$58,MATCH($H42,$A$42:$A$58,0))=0,0,I42/INDEX($E$42:$E$58,MATCH($H42,$A$42:$A$58,0)))</f>
-        <v>52.4026224649165</v>
+        <v>17.4675408216388</v>
       </c>
       <c r="K42" s="16" t="n">
         <f aca="false">C42*G42+I42*INDEX($G$42:$G$58,MATCH($H42,$A$42:$A$58,0))+(F42+J42)*$C$37</f>
-        <v>31399.651380978</v>
+        <v>11654.3432361974</v>
       </c>
       <c r="L42" s="4" t="str">
         <f aca="false">INDEX($B$25:$B$32,MATCH(D42,$A$25:$A$32,0))</f>
@@ -9759,7 +9782,7 @@
       </c>
       <c r="M42" s="4" t="str">
         <f aca="false">INDEX($L$42:$L$58,MATCH($H42,$A$42:$A$58,0))</f>
-        <v>B</v>
+        <v>A</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10576,7 +10599,7 @@
       </c>
       <c r="F59" s="13" t="n">
         <f aca="false">SUM(F42:F58)</f>
-        <v>119.582584827763</v>
+        <v>102.115044006124</v>
       </c>
       <c r="I59" s="13" t="n">
         <f aca="false">SUM(I42:I58)</f>
@@ -10584,14 +10607,14 @@
       </c>
       <c r="J59" s="13" t="n">
         <f aca="false">SUM(J42:J58)</f>
-        <v>142.186276717601</v>
+        <v>107.251195074324</v>
       </c>
       <c r="K59" s="13" t="n">
         <f aca="false">SUM(K42:K58)</f>
-        <v>100078.952067058</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>80333.6439222775</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
         <v>252</v>
       </c>
@@ -10641,7 +10664,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -10684,7 +10707,7 @@
       <c r="B3" s="4"/>
       <c r="C3" s="16" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"A",Recargas!$F$42:$F$58)</f>
-        <v>34.9350816432777</v>
+        <v>17.4675408216388</v>
       </c>
       <c r="D3" s="16" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"B",Recargas!$F$42:$F$58)</f>
@@ -10696,11 +10719,11 @@
       </c>
       <c r="F3" s="16" t="n">
         <f aca="false">SUM(C3:E3)</f>
-        <v>119.582584827763</v>
+        <v>102.115044006125</v>
       </c>
       <c r="G3" s="16" t="n">
         <f aca="false">SUMPRODUCT(Recargas!$C$42:$C$58,Recargas!$G$42:$G$58)+SUM(Recargas!$F$42:$F$58)*Recargas!$C$37</f>
-        <v>38598.4641937406</v>
+        <v>37550.4117444423</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10714,7 +10737,7 @@
       </c>
       <c r="D4" s="13" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"B",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"B",Recargas!$J$42:$J$58)</f>
-        <v>152.025243622599</v>
+        <v>99.6226211576829</v>
       </c>
       <c r="E4" s="13" t="n">
         <f aca="false">SUMIF(Recargas!$L$42:$L$58,"R",Recargas!$F$42:$F$58)+SUMIF(Recargas!$M$42:$M$58,"R",Recargas!$J$42:$J$58)</f>
@@ -10722,11 +10745,11 @@
       </c>
       <c r="F4" s="13" t="n">
         <f aca="false">SUM(C4:E4)</f>
-        <v>261.768861545365</v>
+        <v>209.366239080448</v>
       </c>
       <c r="G4" s="13" t="n">
         <f aca="false">Recargas!K59</f>
-        <v>100078.952067058</v>
+        <v>80333.6439222775</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10764,19 +10787,19 @@
       </c>
       <c r="D7" s="17" t="n">
         <f aca="false">IF(B7=0,0,$F$4/B7)</f>
-        <v>13.7773085023876</v>
+        <v>11.0192757410762</v>
       </c>
       <c r="E7" s="17" t="n">
         <f aca="false">IF(C7=0,0,$G$4/C7)</f>
-        <v>50.039476033529</v>
+        <v>40.1668219611388</v>
       </c>
       <c r="F7" s="18" t="n">
         <f aca="false">MAX(D7,E7)</f>
-        <v>50.039476033529</v>
+        <v>40.1668219611388</v>
       </c>
       <c r="G7" s="18" t="n">
         <f aca="false">F7/Recargas!$C$38</f>
-        <v>10.0078952067058</v>
+        <v>8.03336439222775</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10793,19 +10816,19 @@
       </c>
       <c r="D8" s="17" t="n">
         <f aca="false">IF(B8=0,0,$F$4/B8)</f>
-        <v>43.6281435908941</v>
+        <v>34.8943731800747</v>
       </c>
       <c r="E8" s="17" t="n">
         <f aca="false">IF(C8=0,0,$G$4/C8)</f>
-        <v>16.6798253445097</v>
+        <v>13.3889406537129</v>
       </c>
       <c r="F8" s="18" t="n">
         <f aca="false">MAX(D8,E8)</f>
-        <v>43.6281435908941</v>
+        <v>34.8943731800747</v>
       </c>
       <c r="G8" s="18" t="n">
         <f aca="false">F8/Recargas!$C$38</f>
-        <v>8.72562871817882</v>
+        <v>6.97887463601494</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10822,144 +10845,242 @@
       </c>
       <c r="D9" s="17" t="n">
         <f aca="false">IF(B9=0,0,$F$4/B9)</f>
-        <v>18.6977758246689</v>
+        <v>14.9547313628892</v>
       </c>
       <c r="E9" s="17" t="n">
         <f aca="false">IF(C9=0,0,$G$4/C9)</f>
-        <v>8.33991267225484</v>
+        <v>6.69447032685646</v>
       </c>
       <c r="F9" s="18" t="n">
         <f aca="false">MAX(D9,E9)</f>
-        <v>18.6977758246689</v>
+        <v>14.9547313628892</v>
       </c>
       <c r="G9" s="18" t="n">
         <f aca="false">F9/Recargas!$C$38</f>
-        <v>3.73955516493378</v>
+        <v>2.99094627257783</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="B10" s="22" t="str">
-        <f aca="false">INDEX(A7:A9,MATCH(MIN(F7:F9),F7:F9,0))</f>
-        <v>Sider GyL Full para balancín 7,50 m</v>
-      </c>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="18" t="n">
-        <f aca="false">MIN(F7:F9)</f>
-        <v>18.6977758246689</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <f aca="false">MIN(G7:G9)</f>
-        <v>3.73955516493378</v>
+      <c r="B10" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="22" t="str">
+        <f aca="false">INDEX(A7:A9,MATCH(MIN(F7:F9),F7:F9,0))</f>
+        <v>Sider GyL Full para balancín 7,50 m</v>
+      </c>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="18" t="n">
+        <f aca="false">MIN(F7:F9)</f>
+        <v>14.9547313628892</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <f aca="false">MIN(G7:G9)</f>
+        <v>2.99094627257783</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="13" t="n">
-        <f aca="false">ROUNDUP(G10,0)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="22" t="str">
+        <f aca="false">IF(G11&lt;=G10,"sí","no")</f>
+        <v>sí</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B14" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>255</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>275</v>
       </c>
-      <c r="B14" s="4"/>
-      <c r="C14" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D14" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
         <v>276</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C15" s="16" t="n">
-        <f aca="false">C14*INDEX(Recargas!$C$25:$C$32,MATCH("A 1 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 1 kg",Recargas!$A$42:$A$58,0))</f>
-        <v>1231.2</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
+        <f aca="false">Escenarios!G27/(Datos!$C$4*Recargas!$C$38)</f>
+        <v>412.5265036165</v>
+      </c>
+      <c r="D15" s="17" t="n">
+        <f aca="false">Escenarios!G35/(Datos!$C$4*Recargas!$C$38)</f>
+        <v>0.49330132672877</v>
+      </c>
+      <c r="E15" s="28" t="s">
         <v>277</v>
       </c>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>278</v>
+      </c>
       <c r="B16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="13" t="n">
-        <f aca="false">C15+D14*INDEX(Recargas!$C$25:$C$32,MATCH("B 5 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 5 kg",Recargas!$A$42:$A$58,0))+E14*INDEX(Recargas!$C$25:$C$32,MATCH("R 50 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 50 kg s/ruedas",Recargas!$A$42:$A$58,0))+(C14+D14+E14)*Recargas!$C$37</f>
-        <v>4403.2</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C16" s="16" t="n">
+        <f aca="false">Recargas!C59/Recargas!$C$38</f>
+        <v>953.18546190644</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <f aca="false">MAX(F3/INDEX(B7:B9,MATCH(MIN(F7:F9),F7:F9,0)),G3/INDEX(C7:C9,MATCH(MIN(F7:F9),F7:F9,0)))/Recargas!$C$38</f>
+        <v>1.45878634294464</v>
+      </c>
+      <c r="E16" s="28" t="str">
+        <f aca="false">B11</f>
+        <v>Sider GyL Full para balancín 7,50 m</v>
+      </c>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>278</v>
-      </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="22" t="str">
-        <f aca="false">IF(C16&lt;=F14,"sí","no")</f>
+        <v>261</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="13" t="n">
+        <f aca="false">(Recargas!C59+Recargas!I59)/Recargas!$C$38</f>
+        <v>1906.37092381288</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <f aca="false">G11</f>
+        <v>2.99094627257783</v>
+      </c>
+      <c r="E17" s="29" t="str">
+        <f aca="false">B11</f>
+        <v>Sider GyL Full para balancín 7,50 m</v>
+      </c>
+      <c r="F17" s="29"/>
+      <c r="G17" s="29"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B20" s="4"/>
+      <c r="C20" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="16" t="n">
+        <f aca="false">C20*INDEX(Recargas!$C$25:$C$32,MATCH("A 1 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 1 kg",Recargas!$A$42:$A$58,0))</f>
+        <v>1231.2</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="13" t="n">
+        <f aca="false">C21+D20*INDEX(Recargas!$C$25:$C$32,MATCH("B 5 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 5 kg",Recargas!$A$42:$A$58,0))+E20*INDEX(Recargas!$C$25:$C$32,MATCH("R 50 kg",Recargas!$A$25:$A$32,0))*INDEX(Recargas!$G$42:$G$58,MATCH("ABC 50 kg s/ruedas",Recargas!$A$42:$A$58,0))+(C20+D20+E20)*Recargas!$C$37</f>
+        <v>4403.2</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="22" t="str">
+        <f aca="false">IF(C22&lt;=F20,"sí","no")</f>
         <v>no</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="A19:G19"/>
+  <mergeCells count="5">
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="E15:G15"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="A25:G25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Palletizado: vista superior de los vehículos por escenario
Hoja Vistas y PDF con la carga de cada vehículo en los 5 escenarios:
manuales en el camión chico, rodantes en la Master (por zona), cilindros
de manuales y de rodantes en el sider, y el viaje tipo de recargas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/palletizado_PT.xlsx
+++ b/salida/palletizado_PT.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Escenarios" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Recargas" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Recargas_camion" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Vistas" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="286">
   <si>
     <t xml:space="preserve">General</t>
   </si>
@@ -881,6 +882,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fuentes: Iveco, 9 jaulas A, 8 jaulas B, 2 pallets de rodantes, unas 2 t y pico de 1,2 t (Word Proceso de recargas, Recepción y registro). Camión chico y sider: hojas Datos y Camion. Máximo de 3 viajes por día: dato del usuario.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vista superior de los vehículos por escenario (dibujada con los valores de 2035)</t>
   </si>
 </sst>
 </file>
@@ -1218,6 +1222,196 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>837720</xdr:colOff>
+      <xdr:row>49</xdr:row>
+      <xdr:rowOff>85320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="177840" y="380880"/>
+          <a:ext cx="7238520" cy="9038880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>837720</xdr:colOff>
+      <xdr:row>98</xdr:row>
+      <xdr:rowOff>85680</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="177840" y="9715680"/>
+          <a:ext cx="7238520" cy="9038880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>100</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>837720</xdr:colOff>
+      <xdr:row>147</xdr:row>
+      <xdr:rowOff>85320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 3" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId3"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="177840" y="19050120"/>
+          <a:ext cx="7238520" cy="9038880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>149</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>837720</xdr:colOff>
+      <xdr:row>196</xdr:row>
+      <xdr:rowOff>85320</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 4" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId4"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="177840" y="28384560"/>
+          <a:ext cx="7238520" cy="9038880"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>198</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>837720</xdr:colOff>
+      <xdr:row>209</xdr:row>
+      <xdr:rowOff>56880</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 5" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId5"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="177840" y="37719000"/>
+          <a:ext cx="7238520" cy="2152440"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -11090,4 +11284,33 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>